<commit_message>
additional comments section added
</commit_message>
<xml_diff>
--- a/src/data/TestData.xlsx
+++ b/src/data/TestData.xlsx
@@ -1,12 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="5" lowestEdited="5" rupBuild="9303"/>
-  <workbookPr defaultThemeVersion="164011" filterPrivacy="1"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="29725"/>
+  <workbookPr filterPrivacy="1"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="11_544C5EE8B02CB03631FC9090E0F4C475D5F060AD" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <bookViews>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+  </bookViews>
   <sheets>
-    <sheet sheetId="1" name="01_Policy_Info" state="visible" r:id="rId4"/>
-    <sheet sheetId="2" name="02_WH_Locations" state="visible" r:id="rId5"/>
-    <sheet sheetId="3" name="Test Scenario Details" state="visible" r:id="rId6"/>
+    <sheet name="01_Policy_Info" sheetId="1" r:id="rId1"/>
+    <sheet name="02_WH_Locations" sheetId="2" r:id="rId2"/>
+    <sheet name="Test Scenario Details" sheetId="3" r:id="rId3"/>
   </sheets>
   <calcPr calcId="171027"/>
 </workbook>
@@ -6411,17 +6415,17 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="1">
-    <numFmt numFmtId="164" formatCode="$#,##0.00"/>
+    <numFmt numFmtId="164" formatCode="\$#,##0.00"/>
   </numFmts>
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="2">
     <font>
+      <sz val="11"/>
       <color theme="1"/>
+      <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
-      <sz val="11"/>
-      <name val="Calibri"/>
     </font>
     <font>
       <sz val="11"/>
@@ -6808,23 +6812,23 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:AH83"/>
-  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+  <sheetFormatPr defaultRowHeight="14.4"/>
   <cols>
-    <col min="1" max="1" width="35.285714285714285" customWidth="1"/>
-    <col min="2" max="2" width="27.714285714285715" customWidth="1"/>
-    <col min="3" max="3" width="18.857142857142858" customWidth="1"/>
+    <col min="1" max="1" width="35.33203125" customWidth="1"/>
+    <col min="2" max="2" width="27.6640625" customWidth="1"/>
+    <col min="3" max="3" width="18.88671875" customWidth="1"/>
     <col min="4" max="4" width="16" customWidth="1"/>
-    <col min="5" max="5" width="15.428571428571429" customWidth="1"/>
+    <col min="5" max="5" width="15.44140625" customWidth="1"/>
     <col min="6" max="6" width="22" customWidth="1"/>
-    <col min="7" max="7" width="24.714285714285715" customWidth="1"/>
-    <col min="8" max="8" width="24.428571428571427" customWidth="1"/>
-    <col min="9" max="11" width="42.142857142857146" customWidth="1"/>
+    <col min="7" max="7" width="24.6640625" customWidth="1"/>
+    <col min="8" max="8" width="24.44140625" customWidth="1"/>
+    <col min="9" max="11" width="42.109375" customWidth="1"/>
     <col min="12" max="12" width="38" customWidth="1"/>
     <col min="13" max="13" width="16" customWidth="1"/>
     <col min="14" max="14" width="19" customWidth="1"/>
-    <col min="15" max="15" width="42.142857142857146" customWidth="1"/>
+    <col min="15" max="15" width="42.109375" customWidth="1"/>
     <col min="16" max="17" width="16" customWidth="1"/>
     <col min="18" max="18" width="30" customWidth="1"/>
     <col min="19" max="19" width="20" customWidth="1"/>
@@ -6841,10 +6845,10 @@
     <col min="30" max="31" width="18" customWidth="1"/>
     <col min="32" max="32" width="15" customWidth="1"/>
     <col min="33" max="33" width="13" customWidth="1"/>
-    <col min="34" max="34" width="42.142857142857146" customWidth="1"/>
+    <col min="34" max="34" width="42.109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:34" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:34">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -6948,7 +6952,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="2" spans="1:34" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:34">
       <c r="A2" s="1" t="s">
         <v>34</v>
       </c>
@@ -7048,7 +7052,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="3" spans="1:34" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:34">
       <c r="A3" s="1" t="s">
         <v>58</v>
       </c>
@@ -7152,7 +7156,7 @@
         <v>83</v>
       </c>
     </row>
-    <row r="4" spans="1:34" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:34">
       <c r="A4" s="1" t="s">
         <v>84</v>
       </c>
@@ -7252,7 +7256,7 @@
         <v>103</v>
       </c>
     </row>
-    <row r="5" spans="1:34" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:34">
       <c r="A5" s="1" t="s">
         <v>104</v>
       </c>
@@ -7356,7 +7360,7 @@
         <v>128</v>
       </c>
     </row>
-    <row r="6" spans="1:34" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:34">
       <c r="A6" s="1" t="s">
         <v>129</v>
       </c>
@@ -7456,7 +7460,7 @@
         <v>149</v>
       </c>
     </row>
-    <row r="7" spans="1:34" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:34">
       <c r="A7" s="1" t="s">
         <v>150</v>
       </c>
@@ -7560,7 +7564,7 @@
         <v>174</v>
       </c>
     </row>
-    <row r="8" spans="1:34" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:34">
       <c r="A8" s="1" t="s">
         <v>175</v>
       </c>
@@ -7660,7 +7664,7 @@
         <v>195</v>
       </c>
     </row>
-    <row r="9" spans="1:34" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:34">
       <c r="A9" s="1" t="s">
         <v>196</v>
       </c>
@@ -7764,7 +7768,7 @@
         <v>218</v>
       </c>
     </row>
-    <row r="10" spans="1:34" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:34">
       <c r="A10" s="1" t="s">
         <v>219</v>
       </c>
@@ -7864,7 +7868,7 @@
         <v>239</v>
       </c>
     </row>
-    <row r="11" spans="1:34" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:34">
       <c r="A11" s="1" t="s">
         <v>240</v>
       </c>
@@ -7966,7 +7970,7 @@
         <v>261</v>
       </c>
     </row>
-    <row r="12" spans="1:34" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:34">
       <c r="A12" s="1" t="s">
         <v>262</v>
       </c>
@@ -8066,7 +8070,7 @@
         <v>281</v>
       </c>
     </row>
-    <row r="13" spans="1:34" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:34">
       <c r="A13" s="1" t="s">
         <v>282</v>
       </c>
@@ -8170,7 +8174,7 @@
         <v>305</v>
       </c>
     </row>
-    <row r="14" spans="1:34" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:34">
       <c r="A14" s="1" t="s">
         <v>306</v>
       </c>
@@ -8270,7 +8274,7 @@
         <v>325</v>
       </c>
     </row>
-    <row r="15" spans="1:34" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:34">
       <c r="A15" s="1" t="s">
         <v>326</v>
       </c>
@@ -8374,7 +8378,7 @@
         <v>349</v>
       </c>
     </row>
-    <row r="16" spans="1:34" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:34">
       <c r="A16" s="1" t="s">
         <v>350</v>
       </c>
@@ -8476,7 +8480,7 @@
         <v>370</v>
       </c>
     </row>
-    <row r="17" spans="1:34" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:34">
       <c r="A17" s="1" t="s">
         <v>371</v>
       </c>
@@ -8578,7 +8582,7 @@
         <v>394</v>
       </c>
     </row>
-    <row r="18" spans="1:34" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:34">
       <c r="A18" s="1" t="s">
         <v>395</v>
       </c>
@@ -8680,7 +8684,7 @@
         <v>417</v>
       </c>
     </row>
-    <row r="19" spans="1:34" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:34">
       <c r="A19" s="1" t="s">
         <v>418</v>
       </c>
@@ -8784,7 +8788,7 @@
         <v>441</v>
       </c>
     </row>
-    <row r="20" spans="1:34" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:34">
       <c r="A20" s="1" t="s">
         <v>442</v>
       </c>
@@ -8886,7 +8890,7 @@
         <v>462</v>
       </c>
     </row>
-    <row r="21" spans="1:34" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:34">
       <c r="A21" s="1" t="s">
         <v>463</v>
       </c>
@@ -8988,7 +8992,7 @@
         <v>484</v>
       </c>
     </row>
-    <row r="22" spans="1:34" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:34">
       <c r="A22" s="1" t="s">
         <v>485</v>
       </c>
@@ -9090,7 +9094,7 @@
         <v>504</v>
       </c>
     </row>
-    <row r="23" spans="1:34" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:34">
       <c r="A23" s="1" t="s">
         <v>505</v>
       </c>
@@ -9192,7 +9196,7 @@
         <v>526</v>
       </c>
     </row>
-    <row r="24" spans="1:34" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:34">
       <c r="A24" s="1" t="s">
         <v>527</v>
       </c>
@@ -9294,7 +9298,7 @@
         <v>547</v>
       </c>
     </row>
-    <row r="25" spans="1:34" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:34">
       <c r="A25" s="1" t="s">
         <v>548</v>
       </c>
@@ -9398,7 +9402,7 @@
         <v>567</v>
       </c>
     </row>
-    <row r="26" spans="1:34" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:34">
       <c r="A26" s="1" t="s">
         <v>568</v>
       </c>
@@ -9464,7 +9468,7 @@
         <v>25301</v>
       </c>
       <c r="W26" s="2">
-        <v>0.14</v>
+        <v>0.14000000000000001</v>
       </c>
       <c r="X26" s="1" t="s">
         <v>178</v>
@@ -9500,7 +9504,7 @@
         <v>584</v>
       </c>
     </row>
-    <row r="27" spans="1:34" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:34">
       <c r="A27" s="1" t="s">
         <v>585</v>
       </c>
@@ -9604,7 +9608,7 @@
         <v>604</v>
       </c>
     </row>
-    <row r="28" spans="1:34" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:34">
       <c r="A28" s="1" t="s">
         <v>605</v>
       </c>
@@ -9704,7 +9708,7 @@
         <v>622</v>
       </c>
     </row>
-    <row r="29" spans="1:34" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:34">
       <c r="A29" s="1" t="s">
         <v>623</v>
       </c>
@@ -9806,7 +9810,7 @@
         <v>641</v>
       </c>
     </row>
-    <row r="30" spans="1:34" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:34">
       <c r="A30" s="1" t="s">
         <v>642</v>
       </c>
@@ -9908,7 +9912,7 @@
         <v>659</v>
       </c>
     </row>
-    <row r="31" spans="1:34" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:34">
       <c r="A31" s="1" t="s">
         <v>660</v>
       </c>
@@ -10012,7 +10016,7 @@
         <v>678</v>
       </c>
     </row>
-    <row r="32" spans="1:34" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:34">
       <c r="A32" s="1" t="s">
         <v>679</v>
       </c>
@@ -10116,7 +10120,7 @@
         <v>698</v>
       </c>
     </row>
-    <row r="33" spans="1:34" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:34">
       <c r="A33" s="1" t="s">
         <v>699</v>
       </c>
@@ -10218,7 +10222,7 @@
         <v>717</v>
       </c>
     </row>
-    <row r="34" spans="1:34" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:34">
       <c r="A34" s="1" t="s">
         <v>718</v>
       </c>
@@ -10322,7 +10326,7 @@
         <v>733</v>
       </c>
     </row>
-    <row r="35" spans="1:34" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:34">
       <c r="A35" s="1" t="s">
         <v>734</v>
       </c>
@@ -10424,7 +10428,7 @@
         <v>751</v>
       </c>
     </row>
-    <row r="36" spans="1:34" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:34">
       <c r="A36" s="1" t="s">
         <v>752</v>
       </c>
@@ -10524,7 +10528,7 @@
         <v>768</v>
       </c>
     </row>
-    <row r="37" spans="1:34" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:34">
       <c r="A37" s="1" t="s">
         <v>769</v>
       </c>
@@ -10628,7 +10632,7 @@
         <v>786</v>
       </c>
     </row>
-    <row r="38" spans="1:34" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:34">
       <c r="A38" s="1" t="s">
         <v>787</v>
       </c>
@@ -10728,7 +10732,7 @@
         <v>803</v>
       </c>
     </row>
-    <row r="39" spans="1:34" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:34">
       <c r="A39" s="1" t="s">
         <v>804</v>
       </c>
@@ -10832,7 +10836,7 @@
         <v>820</v>
       </c>
     </row>
-    <row r="40" spans="1:34" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:34">
       <c r="A40" s="1" t="s">
         <v>821</v>
       </c>
@@ -10932,7 +10936,7 @@
         <v>835</v>
       </c>
     </row>
-    <row r="41" spans="1:34" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:34">
       <c r="A41" s="1" t="s">
         <v>836</v>
       </c>
@@ -11036,7 +11040,7 @@
         <v>852</v>
       </c>
     </row>
-    <row r="42" spans="1:34" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:34">
       <c r="A42" s="1" t="s">
         <v>853</v>
       </c>
@@ -11136,7 +11140,7 @@
         <v>868</v>
       </c>
     </row>
-    <row r="43" spans="1:34" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:34">
       <c r="A43" s="1" t="s">
         <v>869</v>
       </c>
@@ -11240,7 +11244,7 @@
         <v>886</v>
       </c>
     </row>
-    <row r="44" spans="1:34" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:34">
       <c r="A44" s="1" t="s">
         <v>887</v>
       </c>
@@ -11340,7 +11344,7 @@
         <v>903</v>
       </c>
     </row>
-    <row r="45" spans="1:34" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:34">
       <c r="A45" s="1" t="s">
         <v>904</v>
       </c>
@@ -11444,7 +11448,7 @@
         <v>920</v>
       </c>
     </row>
-    <row r="46" spans="1:34" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:34">
       <c r="A46" s="1" t="s">
         <v>921</v>
       </c>
@@ -11544,7 +11548,7 @@
         <v>937</v>
       </c>
     </row>
-    <row r="47" spans="1:34" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:34">
       <c r="A47" s="1" t="s">
         <v>938</v>
       </c>
@@ -11648,7 +11652,7 @@
         <v>953</v>
       </c>
     </row>
-    <row r="48" spans="1:34" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:34">
       <c r="A48" s="1" t="s">
         <v>954</v>
       </c>
@@ -11748,7 +11752,7 @@
         <v>970</v>
       </c>
     </row>
-    <row r="49" spans="1:34" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:34">
       <c r="A49" s="1" t="s">
         <v>971</v>
       </c>
@@ -11852,7 +11856,7 @@
         <v>990</v>
       </c>
     </row>
-    <row r="50" spans="1:34" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:34">
       <c r="A50" s="1" t="s">
         <v>991</v>
       </c>
@@ -11954,7 +11958,7 @@
         <v>1007</v>
       </c>
     </row>
-    <row r="51" spans="1:34" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:34">
       <c r="A51" s="1" t="s">
         <v>1008</v>
       </c>
@@ -12056,7 +12060,7 @@
         <v>1024</v>
       </c>
     </row>
-    <row r="52" spans="1:34" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:34">
       <c r="A52" s="1" t="s">
         <v>1025</v>
       </c>
@@ -12156,7 +12160,7 @@
         <v>1041</v>
       </c>
     </row>
-    <row r="53" spans="1:34" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:34">
       <c r="A53" s="1" t="s">
         <v>1042</v>
       </c>
@@ -12260,7 +12264,7 @@
         <v>1061</v>
       </c>
     </row>
-    <row r="54" spans="1:34" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:34">
       <c r="A54" s="1" t="s">
         <v>1062</v>
       </c>
@@ -12360,7 +12364,7 @@
         <v>1079</v>
       </c>
     </row>
-    <row r="55" spans="1:34" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:34">
       <c r="A55" s="1" t="s">
         <v>1080</v>
       </c>
@@ -12464,7 +12468,7 @@
         <v>1098</v>
       </c>
     </row>
-    <row r="56" spans="1:34" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:34">
       <c r="A56" s="1" t="s">
         <v>1099</v>
       </c>
@@ -12568,7 +12572,7 @@
         <v>1115</v>
       </c>
     </row>
-    <row r="57" spans="1:34" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:34">
       <c r="A57" s="1" t="s">
         <v>1116</v>
       </c>
@@ -12668,7 +12672,7 @@
         <v>1134</v>
       </c>
     </row>
-    <row r="58" spans="1:34" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:34">
       <c r="A58" s="1" t="s">
         <v>1135</v>
       </c>
@@ -12768,7 +12772,7 @@
         <v>1154</v>
       </c>
     </row>
-    <row r="59" spans="1:34" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:34">
       <c r="A59" s="1" t="s">
         <v>1155</v>
       </c>
@@ -12870,7 +12874,7 @@
         <v>1173</v>
       </c>
     </row>
-    <row r="60" spans="1:34" x14ac:dyDescent="0.25">
+    <row r="60" spans="1:34">
       <c r="A60" s="1" t="s">
         <v>1174</v>
       </c>
@@ -12972,7 +12976,7 @@
         <v>1192</v>
       </c>
     </row>
-    <row r="61" spans="1:34" x14ac:dyDescent="0.25">
+    <row r="61" spans="1:34">
       <c r="A61" s="1" t="s">
         <v>1193</v>
       </c>
@@ -13076,7 +13080,7 @@
         <v>1211</v>
       </c>
     </row>
-    <row r="62" spans="1:34" x14ac:dyDescent="0.25">
+    <row r="62" spans="1:34">
       <c r="A62" s="1" t="s">
         <v>1212</v>
       </c>
@@ -13176,7 +13180,7 @@
         <v>1227</v>
       </c>
     </row>
-    <row r="63" spans="1:34" x14ac:dyDescent="0.25">
+    <row r="63" spans="1:34">
       <c r="A63" s="1" t="s">
         <v>1228</v>
       </c>
@@ -13280,7 +13284,7 @@
         <v>1246</v>
       </c>
     </row>
-    <row r="64" spans="1:34" x14ac:dyDescent="0.25">
+    <row r="64" spans="1:34">
       <c r="A64" s="1" t="s">
         <v>1247</v>
       </c>
@@ -13380,7 +13384,7 @@
         <v>1266</v>
       </c>
     </row>
-    <row r="65" spans="1:34" x14ac:dyDescent="0.25">
+    <row r="65" spans="1:34">
       <c r="A65" s="1" t="s">
         <v>1267</v>
       </c>
@@ -13484,7 +13488,7 @@
         <v>1283</v>
       </c>
     </row>
-    <row r="66" spans="1:34" x14ac:dyDescent="0.25">
+    <row r="66" spans="1:34">
       <c r="A66" s="1" t="s">
         <v>1284</v>
       </c>
@@ -13586,7 +13590,7 @@
         <v>1301</v>
       </c>
     </row>
-    <row r="67" spans="1:34" x14ac:dyDescent="0.25">
+    <row r="67" spans="1:34">
       <c r="A67" s="1" t="s">
         <v>1302</v>
       </c>
@@ -13688,7 +13692,7 @@
         <v>1318</v>
       </c>
     </row>
-    <row r="68" spans="1:34" x14ac:dyDescent="0.25">
+    <row r="68" spans="1:34">
       <c r="A68" s="1" t="s">
         <v>1319</v>
       </c>
@@ -13790,7 +13794,7 @@
         <v>1337</v>
       </c>
     </row>
-    <row r="69" spans="1:34" x14ac:dyDescent="0.25">
+    <row r="69" spans="1:34">
       <c r="A69" s="1" t="s">
         <v>1338</v>
       </c>
@@ -13894,7 +13898,7 @@
         <v>1357</v>
       </c>
     </row>
-    <row r="70" spans="1:34" x14ac:dyDescent="0.25">
+    <row r="70" spans="1:34">
       <c r="A70" s="1" t="s">
         <v>1358</v>
       </c>
@@ -13994,7 +13998,7 @@
         <v>1374</v>
       </c>
     </row>
-    <row r="71" spans="1:34" x14ac:dyDescent="0.25">
+    <row r="71" spans="1:34">
       <c r="A71" s="1" t="s">
         <v>1375</v>
       </c>
@@ -14098,7 +14102,7 @@
         <v>1391</v>
       </c>
     </row>
-    <row r="72" spans="1:34" x14ac:dyDescent="0.25">
+    <row r="72" spans="1:34">
       <c r="A72" s="1" t="s">
         <v>1392</v>
       </c>
@@ -14200,7 +14204,7 @@
         <v>1408</v>
       </c>
     </row>
-    <row r="73" spans="1:34" x14ac:dyDescent="0.25">
+    <row r="73" spans="1:34">
       <c r="A73" s="1" t="s">
         <v>1409</v>
       </c>
@@ -14304,7 +14308,7 @@
         <v>1426</v>
       </c>
     </row>
-    <row r="74" spans="1:34" x14ac:dyDescent="0.25">
+    <row r="74" spans="1:34">
       <c r="A74" s="1" t="s">
         <v>1427</v>
       </c>
@@ -14404,7 +14408,7 @@
         <v>1441</v>
       </c>
     </row>
-    <row r="75" spans="1:34" x14ac:dyDescent="0.25">
+    <row r="75" spans="1:34">
       <c r="A75" s="1" t="s">
         <v>1442</v>
       </c>
@@ -14506,7 +14510,7 @@
         <v>1456</v>
       </c>
     </row>
-    <row r="76" spans="1:34" x14ac:dyDescent="0.25">
+    <row r="76" spans="1:34">
       <c r="A76" s="1" t="s">
         <v>1457</v>
       </c>
@@ -14608,7 +14612,7 @@
         <v>1473</v>
       </c>
     </row>
-    <row r="77" spans="1:34" x14ac:dyDescent="0.25">
+    <row r="77" spans="1:34">
       <c r="A77" s="1" t="s">
         <v>1474</v>
       </c>
@@ -14712,7 +14716,7 @@
         <v>1491</v>
       </c>
     </row>
-    <row r="78" spans="1:34" x14ac:dyDescent="0.25">
+    <row r="78" spans="1:34">
       <c r="A78" s="1" t="s">
         <v>1492</v>
       </c>
@@ -14812,7 +14816,7 @@
         <v>1507</v>
       </c>
     </row>
-    <row r="79" spans="1:34" x14ac:dyDescent="0.25">
+    <row r="79" spans="1:34">
       <c r="A79" s="1" t="s">
         <v>1508</v>
       </c>
@@ -14916,7 +14920,7 @@
         <v>1522</v>
       </c>
     </row>
-    <row r="80" spans="1:34" x14ac:dyDescent="0.25">
+    <row r="80" spans="1:34">
       <c r="A80" s="1" t="s">
         <v>1523</v>
       </c>
@@ -15018,7 +15022,7 @@
         <v>1537</v>
       </c>
     </row>
-    <row r="81" spans="1:34" x14ac:dyDescent="0.25">
+    <row r="81" spans="1:34">
       <c r="A81" s="1" t="s">
         <v>1538</v>
       </c>
@@ -15122,7 +15126,7 @@
         <v>1556</v>
       </c>
     </row>
-    <row r="82" spans="1:34" x14ac:dyDescent="0.25">
+    <row r="82" spans="1:34">
       <c r="A82" s="1" t="s">
         <v>1557</v>
       </c>
@@ -15226,7 +15230,7 @@
         <v>1573</v>
       </c>
     </row>
-    <row r="83" spans="1:34" x14ac:dyDescent="0.25">
+    <row r="83" spans="1:34">
       <c r="A83" s="1" t="s">
         <v>1574</v>
       </c>
@@ -15329,28 +15333,28 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:AH1"/>
+  <autoFilter ref="A1:AH1" xr:uid="{00000000-0009-0000-0000-000000000000}"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:W331"/>
-  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+  <sheetFormatPr defaultRowHeight="14.4"/>
   <cols>
-    <col min="1" max="2" width="9.285714285714286" customWidth="1"/>
+    <col min="1" max="2" width="9.33203125" customWidth="1"/>
     <col min="3" max="3" width="27" customWidth="1"/>
     <col min="4" max="5" width="18" customWidth="1"/>
-    <col min="6" max="7" width="9.285714285714286" customWidth="1"/>
+    <col min="6" max="7" width="9.33203125" customWidth="1"/>
     <col min="8" max="8" width="25" customWidth="1"/>
     <col min="9" max="10" width="20" customWidth="1"/>
     <col min="11" max="11" width="24" customWidth="1"/>
     <col min="12" max="12" width="26" customWidth="1"/>
     <col min="13" max="13" width="20" customWidth="1"/>
-    <col min="14" max="14" width="26.428571428571427" customWidth="1"/>
-    <col min="15" max="15" width="42.142857142857146" customWidth="1"/>
+    <col min="14" max="14" width="26.44140625" customWidth="1"/>
+    <col min="15" max="15" width="42.109375" customWidth="1"/>
     <col min="16" max="16" width="22" customWidth="1"/>
     <col min="17" max="17" width="26" customWidth="1"/>
     <col min="18" max="18" width="19" customWidth="1"/>
@@ -15359,10 +15363,10 @@
     <col min="21" max="21" width="13" customWidth="1"/>
     <col min="22" max="22" width="12" customWidth="1"/>
     <col min="23" max="23" width="18" customWidth="1"/>
-    <col min="24" max="24" width="13.571428571428571" customWidth="1"/>
+    <col min="24" max="24" width="13.5546875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:23">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -15433,7 +15437,7 @@
         <v>1609</v>
       </c>
     </row>
-    <row r="2" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:23">
       <c r="A2" s="1" t="s">
         <v>34</v>
       </c>
@@ -15504,7 +15508,7 @@
         <v>1619</v>
       </c>
     </row>
-    <row r="3" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:23">
       <c r="A3" s="1" t="s">
         <v>34</v>
       </c>
@@ -15573,7 +15577,7 @@
         <v>1617</v>
       </c>
     </row>
-    <row r="4" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:23">
       <c r="A4" s="1" t="s">
         <v>34</v>
       </c>
@@ -15642,7 +15646,7 @@
         <v>1619</v>
       </c>
     </row>
-    <row r="5" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:23">
       <c r="A5" s="1" t="s">
         <v>34</v>
       </c>
@@ -15713,7 +15717,7 @@
         <v>1619</v>
       </c>
     </row>
-    <row r="6" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:23">
       <c r="A6" s="1" t="s">
         <v>58</v>
       </c>
@@ -15784,7 +15788,7 @@
         <v>1619</v>
       </c>
     </row>
-    <row r="7" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:23">
       <c r="A7" s="1" t="s">
         <v>58</v>
       </c>
@@ -15853,7 +15857,7 @@
         <v>1617</v>
       </c>
     </row>
-    <row r="8" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:23">
       <c r="A8" s="1" t="s">
         <v>84</v>
       </c>
@@ -15920,7 +15924,7 @@
         <v>1619</v>
       </c>
     </row>
-    <row r="9" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:23">
       <c r="A9" s="1" t="s">
         <v>104</v>
       </c>
@@ -15991,7 +15995,7 @@
         <v>1619</v>
       </c>
     </row>
-    <row r="10" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:23">
       <c r="A10" s="1" t="s">
         <v>104</v>
       </c>
@@ -16060,7 +16064,7 @@
         <v>1619</v>
       </c>
     </row>
-    <row r="11" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:23">
       <c r="A11" s="1" t="s">
         <v>129</v>
       </c>
@@ -16101,7 +16105,7 @@
         <v>1614</v>
       </c>
       <c r="N11" s="1">
-        <v>0.14</v>
+        <v>0.14000000000000001</v>
       </c>
       <c r="O11" s="1" t="s">
         <v>1655</v>
@@ -16129,7 +16133,7 @@
         <v>1619</v>
       </c>
     </row>
-    <row r="12" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:23">
       <c r="A12" s="1" t="s">
         <v>150</v>
       </c>
@@ -16198,7 +16202,7 @@
         <v>1619</v>
       </c>
     </row>
-    <row r="13" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:23">
       <c r="A13" s="1" t="s">
         <v>150</v>
       </c>
@@ -16269,7 +16273,7 @@
         <v>1617</v>
       </c>
     </row>
-    <row r="14" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:23">
       <c r="A14" s="1" t="s">
         <v>150</v>
       </c>
@@ -16338,7 +16342,7 @@
         <v>1619</v>
       </c>
     </row>
-    <row r="15" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:23">
       <c r="A15" s="1" t="s">
         <v>150</v>
       </c>
@@ -16407,7 +16411,7 @@
         <v>1619</v>
       </c>
     </row>
-    <row r="16" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:23">
       <c r="A16" s="1" t="s">
         <v>150</v>
       </c>
@@ -16476,7 +16480,7 @@
         <v>1619</v>
       </c>
     </row>
-    <row r="17" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:23">
       <c r="A17" s="1" t="s">
         <v>150</v>
       </c>
@@ -16517,7 +16521,7 @@
         <v>1630</v>
       </c>
       <c r="N17" s="1">
-        <v>0.57</v>
+        <v>0.56999999999999995</v>
       </c>
       <c r="O17" s="1" t="s">
         <v>1685</v>
@@ -16547,7 +16551,7 @@
         <v>1619</v>
       </c>
     </row>
-    <row r="18" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:23">
       <c r="A18" s="1" t="s">
         <v>150</v>
       </c>
@@ -16616,7 +16620,7 @@
         <v>1619</v>
       </c>
     </row>
-    <row r="19" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:23">
       <c r="A19" s="1" t="s">
         <v>150</v>
       </c>
@@ -16685,7 +16689,7 @@
         <v>1617</v>
       </c>
     </row>
-    <row r="20" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:23">
       <c r="A20" s="1" t="s">
         <v>150</v>
       </c>
@@ -16756,7 +16760,7 @@
         <v>1619</v>
       </c>
     </row>
-    <row r="21" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:23">
       <c r="A21" s="1" t="s">
         <v>150</v>
       </c>
@@ -16825,7 +16829,7 @@
         <v>1619</v>
       </c>
     </row>
-    <row r="22" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:23">
       <c r="A22" s="1" t="s">
         <v>175</v>
       </c>
@@ -16896,7 +16900,7 @@
         <v>1619</v>
       </c>
     </row>
-    <row r="23" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:23">
       <c r="A23" s="1" t="s">
         <v>175</v>
       </c>
@@ -16965,7 +16969,7 @@
         <v>1619</v>
       </c>
     </row>
-    <row r="24" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:23">
       <c r="A24" s="1" t="s">
         <v>175</v>
       </c>
@@ -17032,7 +17036,7 @@
         <v>1617</v>
       </c>
     </row>
-    <row r="25" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:23">
       <c r="A25" s="1" t="s">
         <v>175</v>
       </c>
@@ -17103,7 +17107,7 @@
         <v>1619</v>
       </c>
     </row>
-    <row r="26" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:23">
       <c r="A26" s="1" t="s">
         <v>175</v>
       </c>
@@ -17172,7 +17176,7 @@
         <v>1617</v>
       </c>
     </row>
-    <row r="27" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:23">
       <c r="A27" s="1" t="s">
         <v>175</v>
       </c>
@@ -17241,7 +17245,7 @@
         <v>1619</v>
       </c>
     </row>
-    <row r="28" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:23">
       <c r="A28" s="1" t="s">
         <v>175</v>
       </c>
@@ -17310,7 +17314,7 @@
         <v>1619</v>
       </c>
     </row>
-    <row r="29" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:23">
       <c r="A29" s="1" t="s">
         <v>175</v>
       </c>
@@ -17379,7 +17383,7 @@
         <v>1617</v>
       </c>
     </row>
-    <row r="30" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:23">
       <c r="A30" s="1" t="s">
         <v>175</v>
       </c>
@@ -17448,7 +17452,7 @@
         <v>1619</v>
       </c>
     </row>
-    <row r="31" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:23">
       <c r="A31" s="1" t="s">
         <v>175</v>
       </c>
@@ -17519,7 +17523,7 @@
         <v>1619</v>
       </c>
     </row>
-    <row r="32" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:23">
       <c r="A32" s="1" t="s">
         <v>196</v>
       </c>
@@ -17586,7 +17590,7 @@
         <v>1617</v>
       </c>
     </row>
-    <row r="33" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:23">
       <c r="A33" s="1" t="s">
         <v>196</v>
       </c>
@@ -17625,7 +17629,7 @@
         <v>1614</v>
       </c>
       <c r="N33" s="1">
-        <v>0.57</v>
+        <v>0.56999999999999995</v>
       </c>
       <c r="O33" s="1" t="s">
         <v>1643</v>
@@ -17653,7 +17657,7 @@
         <v>1619</v>
       </c>
     </row>
-    <row r="34" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:23">
       <c r="A34" s="1" t="s">
         <v>196</v>
       </c>
@@ -17722,7 +17726,7 @@
         <v>1617</v>
       </c>
     </row>
-    <row r="35" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:23">
       <c r="A35" s="1" t="s">
         <v>196</v>
       </c>
@@ -17793,7 +17797,7 @@
         <v>1619</v>
       </c>
     </row>
-    <row r="36" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:23">
       <c r="A36" s="1" t="s">
         <v>219</v>
       </c>
@@ -17862,7 +17866,7 @@
         <v>1619</v>
       </c>
     </row>
-    <row r="37" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:23">
       <c r="A37" s="1" t="s">
         <v>219</v>
       </c>
@@ -17903,7 +17907,7 @@
         <v>1642</v>
       </c>
       <c r="N37" s="1">
-        <v>0.57</v>
+        <v>0.56999999999999995</v>
       </c>
       <c r="O37" s="1" t="s">
         <v>1767</v>
@@ -17931,7 +17935,7 @@
         <v>1617</v>
       </c>
     </row>
-    <row r="38" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:23">
       <c r="A38" s="1" t="s">
         <v>219</v>
       </c>
@@ -18002,7 +18006,7 @@
         <v>1619</v>
       </c>
     </row>
-    <row r="39" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:23">
       <c r="A39" s="1" t="s">
         <v>219</v>
       </c>
@@ -18073,7 +18077,7 @@
         <v>1619</v>
       </c>
     </row>
-    <row r="40" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:23">
       <c r="A40" s="1" t="s">
         <v>240</v>
       </c>
@@ -18142,7 +18146,7 @@
         <v>1617</v>
       </c>
     </row>
-    <row r="41" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:23">
       <c r="A41" s="1" t="s">
         <v>240</v>
       </c>
@@ -18213,7 +18217,7 @@
         <v>1619</v>
       </c>
     </row>
-    <row r="42" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:23">
       <c r="A42" s="1" t="s">
         <v>240</v>
       </c>
@@ -18284,7 +18288,7 @@
         <v>1619</v>
       </c>
     </row>
-    <row r="43" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:23">
       <c r="A43" s="1" t="s">
         <v>240</v>
       </c>
@@ -18353,7 +18357,7 @@
         <v>1619</v>
       </c>
     </row>
-    <row r="44" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:23">
       <c r="A44" s="1" t="s">
         <v>262</v>
       </c>
@@ -18422,7 +18426,7 @@
         <v>1619</v>
       </c>
     </row>
-    <row r="45" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:23">
       <c r="A45" s="1" t="s">
         <v>262</v>
       </c>
@@ -18493,7 +18497,7 @@
         <v>1619</v>
       </c>
     </row>
-    <row r="46" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:23">
       <c r="A46" s="1" t="s">
         <v>262</v>
       </c>
@@ -18562,7 +18566,7 @@
         <v>1619</v>
       </c>
     </row>
-    <row r="47" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:23">
       <c r="A47" s="1" t="s">
         <v>262</v>
       </c>
@@ -18631,7 +18635,7 @@
         <v>1617</v>
       </c>
     </row>
-    <row r="48" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:23">
       <c r="A48" s="1" t="s">
         <v>282</v>
       </c>
@@ -18670,7 +18674,7 @@
         <v>1630</v>
       </c>
       <c r="N48" s="1">
-        <v>0.28</v>
+        <v>0.28000000000000003</v>
       </c>
       <c r="O48" s="1" t="s">
         <v>1806</v>
@@ -18700,7 +18704,7 @@
         <v>1619</v>
       </c>
     </row>
-    <row r="49" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:23">
       <c r="A49" s="1" t="s">
         <v>282</v>
       </c>
@@ -18769,7 +18773,7 @@
         <v>1619</v>
       </c>
     </row>
-    <row r="50" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:23">
       <c r="A50" s="1" t="s">
         <v>282</v>
       </c>
@@ -18838,7 +18842,7 @@
         <v>1617</v>
       </c>
     </row>
-    <row r="51" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:23">
       <c r="A51" s="1" t="s">
         <v>282</v>
       </c>
@@ -18909,7 +18913,7 @@
         <v>1619</v>
       </c>
     </row>
-    <row r="52" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:23">
       <c r="A52" s="1" t="s">
         <v>306</v>
       </c>
@@ -18978,7 +18982,7 @@
         <v>1617</v>
       </c>
     </row>
-    <row r="53" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:23">
       <c r="A53" s="1" t="s">
         <v>306</v>
       </c>
@@ -19047,7 +19051,7 @@
         <v>1617</v>
       </c>
     </row>
-    <row r="54" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:23">
       <c r="A54" s="1" t="s">
         <v>306</v>
       </c>
@@ -19118,7 +19122,7 @@
         <v>1619</v>
       </c>
     </row>
-    <row r="55" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:23">
       <c r="A55" s="1" t="s">
         <v>306</v>
       </c>
@@ -19187,7 +19191,7 @@
         <v>1619</v>
       </c>
     </row>
-    <row r="56" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:23">
       <c r="A56" s="1" t="s">
         <v>326</v>
       </c>
@@ -19258,7 +19262,7 @@
         <v>1619</v>
       </c>
     </row>
-    <row r="57" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:23">
       <c r="A57" s="1" t="s">
         <v>326</v>
       </c>
@@ -19329,7 +19333,7 @@
         <v>1619</v>
       </c>
     </row>
-    <row r="58" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:23">
       <c r="A58" s="1" t="s">
         <v>326</v>
       </c>
@@ -19398,7 +19402,7 @@
         <v>1619</v>
       </c>
     </row>
-    <row r="59" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:23">
       <c r="A59" s="1" t="s">
         <v>326</v>
       </c>
@@ -19467,7 +19471,7 @@
         <v>1619</v>
       </c>
     </row>
-    <row r="60" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="60" spans="1:23">
       <c r="A60" s="1" t="s">
         <v>350</v>
       </c>
@@ -19534,7 +19538,7 @@
         <v>1619</v>
       </c>
     </row>
-    <row r="61" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="61" spans="1:23">
       <c r="A61" s="1" t="s">
         <v>350</v>
       </c>
@@ -19575,7 +19579,7 @@
         <v>1642</v>
       </c>
       <c r="N61" s="1">
-        <v>0.56</v>
+        <v>0.56000000000000005</v>
       </c>
       <c r="O61" s="1" t="s">
         <v>1655</v>
@@ -19603,7 +19607,7 @@
         <v>1619</v>
       </c>
     </row>
-    <row r="62" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="62" spans="1:23">
       <c r="A62" s="1" t="s">
         <v>350</v>
       </c>
@@ -19672,7 +19676,7 @@
         <v>1619</v>
       </c>
     </row>
-    <row r="63" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="63" spans="1:23">
       <c r="A63" s="1" t="s">
         <v>350</v>
       </c>
@@ -19743,7 +19747,7 @@
         <v>1617</v>
       </c>
     </row>
-    <row r="64" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="64" spans="1:23">
       <c r="A64" s="1" t="s">
         <v>371</v>
       </c>
@@ -19812,7 +19816,7 @@
         <v>1619</v>
       </c>
     </row>
-    <row r="65" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="65" spans="1:23">
       <c r="A65" s="1" t="s">
         <v>371</v>
       </c>
@@ -19881,7 +19885,7 @@
         <v>1619</v>
       </c>
     </row>
-    <row r="66" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="66" spans="1:23">
       <c r="A66" s="1" t="s">
         <v>371</v>
       </c>
@@ -19952,7 +19956,7 @@
         <v>1617</v>
       </c>
     </row>
-    <row r="67" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="67" spans="1:23">
       <c r="A67" s="1" t="s">
         <v>371</v>
       </c>
@@ -20021,7 +20025,7 @@
         <v>1619</v>
       </c>
     </row>
-    <row r="68" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="68" spans="1:23">
       <c r="A68" s="1" t="s">
         <v>395</v>
       </c>
@@ -20090,7 +20094,7 @@
         <v>1619</v>
       </c>
     </row>
-    <row r="69" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="69" spans="1:23">
       <c r="A69" s="1" t="s">
         <v>395</v>
       </c>
@@ -20161,7 +20165,7 @@
         <v>1617</v>
       </c>
     </row>
-    <row r="70" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="70" spans="1:23">
       <c r="A70" s="1" t="s">
         <v>395</v>
       </c>
@@ -20230,7 +20234,7 @@
         <v>1619</v>
       </c>
     </row>
-    <row r="71" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="71" spans="1:23">
       <c r="A71" s="1" t="s">
         <v>395</v>
       </c>
@@ -20301,7 +20305,7 @@
         <v>1619</v>
       </c>
     </row>
-    <row r="72" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="72" spans="1:23">
       <c r="A72" s="1" t="s">
         <v>418</v>
       </c>
@@ -20370,7 +20374,7 @@
         <v>1619</v>
       </c>
     </row>
-    <row r="73" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="73" spans="1:23">
       <c r="A73" s="1" t="s">
         <v>418</v>
       </c>
@@ -20439,7 +20443,7 @@
         <v>1619</v>
       </c>
     </row>
-    <row r="74" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="74" spans="1:23">
       <c r="A74" s="1" t="s">
         <v>418</v>
       </c>
@@ -20510,7 +20514,7 @@
         <v>1619</v>
       </c>
     </row>
-    <row r="75" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="75" spans="1:23">
       <c r="A75" s="1" t="s">
         <v>418</v>
       </c>
@@ -20579,7 +20583,7 @@
         <v>1619</v>
       </c>
     </row>
-    <row r="76" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="76" spans="1:23">
       <c r="A76" s="1" t="s">
         <v>442</v>
       </c>
@@ -20648,7 +20652,7 @@
         <v>1619</v>
       </c>
     </row>
-    <row r="77" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="77" spans="1:23">
       <c r="A77" s="1" t="s">
         <v>442</v>
       </c>
@@ -20719,7 +20723,7 @@
         <v>1619</v>
       </c>
     </row>
-    <row r="78" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="78" spans="1:23">
       <c r="A78" s="1" t="s">
         <v>442</v>
       </c>
@@ -20788,7 +20792,7 @@
         <v>1619</v>
       </c>
     </row>
-    <row r="79" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="79" spans="1:23">
       <c r="A79" s="1" t="s">
         <v>442</v>
       </c>
@@ -20859,7 +20863,7 @@
         <v>1617</v>
       </c>
     </row>
-    <row r="80" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="80" spans="1:23">
       <c r="A80" s="1" t="s">
         <v>463</v>
       </c>
@@ -20930,7 +20934,7 @@
         <v>1617</v>
       </c>
     </row>
-    <row r="81" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="81" spans="1:23">
       <c r="A81" s="1" t="s">
         <v>463</v>
       </c>
@@ -20971,7 +20975,7 @@
         <v>1614</v>
       </c>
       <c r="N81" s="1">
-        <v>0.55</v>
+        <v>0.55000000000000004</v>
       </c>
       <c r="O81" s="1" t="s">
         <v>1659</v>
@@ -20999,7 +21003,7 @@
         <v>1619</v>
       </c>
     </row>
-    <row r="82" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="82" spans="1:23">
       <c r="A82" s="1" t="s">
         <v>463</v>
       </c>
@@ -21070,7 +21074,7 @@
         <v>1617</v>
       </c>
     </row>
-    <row r="83" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="83" spans="1:23">
       <c r="A83" s="1" t="s">
         <v>463</v>
       </c>
@@ -21139,7 +21143,7 @@
         <v>1619</v>
       </c>
     </row>
-    <row r="84" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="84" spans="1:23">
       <c r="A84" s="1" t="s">
         <v>485</v>
       </c>
@@ -21206,7 +21210,7 @@
         <v>1619</v>
       </c>
     </row>
-    <row r="85" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="85" spans="1:23">
       <c r="A85" s="1" t="s">
         <v>485</v>
       </c>
@@ -21277,7 +21281,7 @@
         <v>1617</v>
       </c>
     </row>
-    <row r="86" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="86" spans="1:23">
       <c r="A86" s="1" t="s">
         <v>485</v>
       </c>
@@ -21346,7 +21350,7 @@
         <v>1619</v>
       </c>
     </row>
-    <row r="87" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="87" spans="1:23">
       <c r="A87" s="1" t="s">
         <v>485</v>
       </c>
@@ -21415,7 +21419,7 @@
         <v>1619</v>
       </c>
     </row>
-    <row r="88" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="88" spans="1:23">
       <c r="A88" s="1" t="s">
         <v>505</v>
       </c>
@@ -21482,7 +21486,7 @@
         <v>1619</v>
       </c>
     </row>
-    <row r="89" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="89" spans="1:23">
       <c r="A89" s="1" t="s">
         <v>505</v>
       </c>
@@ -21551,7 +21555,7 @@
         <v>1619</v>
       </c>
     </row>
-    <row r="90" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="90" spans="1:23">
       <c r="A90" s="1" t="s">
         <v>505</v>
       </c>
@@ -21620,7 +21624,7 @@
         <v>1619</v>
       </c>
     </row>
-    <row r="91" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="91" spans="1:23">
       <c r="A91" s="1" t="s">
         <v>505</v>
       </c>
@@ -21689,7 +21693,7 @@
         <v>1619</v>
       </c>
     </row>
-    <row r="92" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="92" spans="1:23">
       <c r="A92" s="1" t="s">
         <v>527</v>
       </c>
@@ -21758,7 +21762,7 @@
         <v>1619</v>
       </c>
     </row>
-    <row r="93" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="93" spans="1:23">
       <c r="A93" s="1" t="s">
         <v>527</v>
       </c>
@@ -21827,7 +21831,7 @@
         <v>1619</v>
       </c>
     </row>
-    <row r="94" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="94" spans="1:23">
       <c r="A94" s="1" t="s">
         <v>527</v>
       </c>
@@ -21896,7 +21900,7 @@
         <v>1619</v>
       </c>
     </row>
-    <row r="95" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="95" spans="1:23">
       <c r="A95" s="1" t="s">
         <v>527</v>
       </c>
@@ -21967,7 +21971,7 @@
         <v>1619</v>
       </c>
     </row>
-    <row r="96" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="96" spans="1:23">
       <c r="A96" s="1" t="s">
         <v>548</v>
       </c>
@@ -22038,7 +22042,7 @@
         <v>1619</v>
       </c>
     </row>
-    <row r="97" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="97" spans="1:23">
       <c r="A97" s="1" t="s">
         <v>548</v>
       </c>
@@ -22107,7 +22111,7 @@
         <v>1619</v>
       </c>
     </row>
-    <row r="98" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="98" spans="1:23">
       <c r="A98" s="1" t="s">
         <v>548</v>
       </c>
@@ -22178,7 +22182,7 @@
         <v>1619</v>
       </c>
     </row>
-    <row r="99" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="99" spans="1:23">
       <c r="A99" s="1" t="s">
         <v>548</v>
       </c>
@@ -22247,7 +22251,7 @@
         <v>1619</v>
       </c>
     </row>
-    <row r="100" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="100" spans="1:23">
       <c r="A100" s="1" t="s">
         <v>568</v>
       </c>
@@ -22314,7 +22318,7 @@
         <v>1619</v>
       </c>
     </row>
-    <row r="101" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="101" spans="1:23">
       <c r="A101" s="1" t="s">
         <v>568</v>
       </c>
@@ -22385,7 +22389,7 @@
         <v>1619</v>
       </c>
     </row>
-    <row r="102" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="102" spans="1:23">
       <c r="A102" s="1" t="s">
         <v>568</v>
       </c>
@@ -22454,7 +22458,7 @@
         <v>1619</v>
       </c>
     </row>
-    <row r="103" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="103" spans="1:23">
       <c r="A103" s="1" t="s">
         <v>568</v>
       </c>
@@ -22523,7 +22527,7 @@
         <v>1617</v>
       </c>
     </row>
-    <row r="104" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="104" spans="1:23">
       <c r="A104" s="1" t="s">
         <v>585</v>
       </c>
@@ -22562,7 +22566,7 @@
         <v>1630</v>
       </c>
       <c r="N104" s="1">
-        <v>0.58</v>
+        <v>0.57999999999999996</v>
       </c>
       <c r="O104" s="1" t="s">
         <v>1909</v>
@@ -22590,7 +22594,7 @@
         <v>1617</v>
       </c>
     </row>
-    <row r="105" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="105" spans="1:23">
       <c r="A105" s="1" t="s">
         <v>585</v>
       </c>
@@ -22659,7 +22663,7 @@
         <v>1619</v>
       </c>
     </row>
-    <row r="106" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="106" spans="1:23">
       <c r="A106" s="1" t="s">
         <v>585</v>
       </c>
@@ -22728,7 +22732,7 @@
         <v>1617</v>
       </c>
     </row>
-    <row r="107" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="107" spans="1:23">
       <c r="A107" s="1" t="s">
         <v>585</v>
       </c>
@@ -22799,7 +22803,7 @@
         <v>1619</v>
       </c>
     </row>
-    <row r="108" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="108" spans="1:23">
       <c r="A108" s="1" t="s">
         <v>605</v>
       </c>
@@ -22868,7 +22872,7 @@
         <v>1619</v>
       </c>
     </row>
-    <row r="109" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="109" spans="1:23">
       <c r="A109" s="1" t="s">
         <v>605</v>
       </c>
@@ -22937,7 +22941,7 @@
         <v>1617</v>
       </c>
     </row>
-    <row r="110" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="110" spans="1:23">
       <c r="A110" s="1" t="s">
         <v>605</v>
       </c>
@@ -23008,7 +23012,7 @@
         <v>1619</v>
       </c>
     </row>
-    <row r="111" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="111" spans="1:23">
       <c r="A111" s="1" t="s">
         <v>605</v>
       </c>
@@ -23077,7 +23081,7 @@
         <v>1619</v>
       </c>
     </row>
-    <row r="112" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="112" spans="1:23">
       <c r="A112" s="1" t="s">
         <v>623</v>
       </c>
@@ -23148,7 +23152,7 @@
         <v>1619</v>
       </c>
     </row>
-    <row r="113" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="113" spans="1:23">
       <c r="A113" s="1" t="s">
         <v>623</v>
       </c>
@@ -23219,7 +23223,7 @@
         <v>1619</v>
       </c>
     </row>
-    <row r="114" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="114" spans="1:23">
       <c r="A114" s="1" t="s">
         <v>623</v>
       </c>
@@ -23288,7 +23292,7 @@
         <v>1619</v>
       </c>
     </row>
-    <row r="115" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="115" spans="1:23">
       <c r="A115" s="1" t="s">
         <v>623</v>
       </c>
@@ -23359,7 +23363,7 @@
         <v>1619</v>
       </c>
     </row>
-    <row r="116" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="116" spans="1:23">
       <c r="A116" s="1" t="s">
         <v>642</v>
       </c>
@@ -23426,7 +23430,7 @@
         <v>1619</v>
       </c>
     </row>
-    <row r="117" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="117" spans="1:23">
       <c r="A117" s="1" t="s">
         <v>642</v>
       </c>
@@ -23495,7 +23499,7 @@
         <v>1619</v>
       </c>
     </row>
-    <row r="118" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="118" spans="1:23">
       <c r="A118" s="1" t="s">
         <v>642</v>
       </c>
@@ -23566,7 +23570,7 @@
         <v>1619</v>
       </c>
     </row>
-    <row r="119" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="119" spans="1:23">
       <c r="A119" s="1" t="s">
         <v>642</v>
       </c>
@@ -23635,7 +23639,7 @@
         <v>1619</v>
       </c>
     </row>
-    <row r="120" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="120" spans="1:23">
       <c r="A120" s="1" t="s">
         <v>660</v>
       </c>
@@ -23676,7 +23680,7 @@
         <v>1614</v>
       </c>
       <c r="N120" s="1">
-        <v>0.14</v>
+        <v>0.14000000000000001</v>
       </c>
       <c r="O120" s="1" t="s">
         <v>1925</v>
@@ -23704,7 +23708,7 @@
         <v>1619</v>
       </c>
     </row>
-    <row r="121" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="121" spans="1:23">
       <c r="A121" s="1" t="s">
         <v>660</v>
       </c>
@@ -23775,7 +23779,7 @@
         <v>1619</v>
       </c>
     </row>
-    <row r="122" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="122" spans="1:23">
       <c r="A122" s="1" t="s">
         <v>660</v>
       </c>
@@ -23844,7 +23848,7 @@
         <v>1619</v>
       </c>
     </row>
-    <row r="123" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="123" spans="1:23">
       <c r="A123" s="1" t="s">
         <v>660</v>
       </c>
@@ -23911,7 +23915,7 @@
         <v>1617</v>
       </c>
     </row>
-    <row r="124" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="124" spans="1:23">
       <c r="A124" s="1" t="s">
         <v>679</v>
       </c>
@@ -23978,7 +23982,7 @@
         <v>1617</v>
       </c>
     </row>
-    <row r="125" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="125" spans="1:23">
       <c r="A125" s="1" t="s">
         <v>679</v>
       </c>
@@ -24047,7 +24051,7 @@
         <v>1619</v>
       </c>
     </row>
-    <row r="126" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="126" spans="1:23">
       <c r="A126" s="1" t="s">
         <v>679</v>
       </c>
@@ -24114,7 +24118,7 @@
         <v>1617</v>
       </c>
     </row>
-    <row r="127" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="127" spans="1:23">
       <c r="A127" s="1" t="s">
         <v>679</v>
       </c>
@@ -24185,7 +24189,7 @@
         <v>1619</v>
       </c>
     </row>
-    <row r="128" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="128" spans="1:23">
       <c r="A128" s="1" t="s">
         <v>699</v>
       </c>
@@ -24256,7 +24260,7 @@
         <v>1619</v>
       </c>
     </row>
-    <row r="129" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="129" spans="1:23">
       <c r="A129" s="1" t="s">
         <v>699</v>
       </c>
@@ -24323,7 +24327,7 @@
         <v>1617</v>
       </c>
     </row>
-    <row r="130" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="130" spans="1:23">
       <c r="A130" s="1" t="s">
         <v>699</v>
       </c>
@@ -24394,7 +24398,7 @@
         <v>1619</v>
       </c>
     </row>
-    <row r="131" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="131" spans="1:23">
       <c r="A131" s="1" t="s">
         <v>699</v>
       </c>
@@ -24463,7 +24467,7 @@
         <v>1617</v>
       </c>
     </row>
-    <row r="132" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="132" spans="1:23">
       <c r="A132" s="1" t="s">
         <v>718</v>
       </c>
@@ -24530,7 +24534,7 @@
         <v>1619</v>
       </c>
     </row>
-    <row r="133" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="133" spans="1:23">
       <c r="A133" s="1" t="s">
         <v>718</v>
       </c>
@@ -24601,7 +24605,7 @@
         <v>1619</v>
       </c>
     </row>
-    <row r="134" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="134" spans="1:23">
       <c r="A134" s="1" t="s">
         <v>718</v>
       </c>
@@ -24642,7 +24646,7 @@
         <v>1630</v>
       </c>
       <c r="N134" s="1">
-        <v>0.56</v>
+        <v>0.56000000000000005</v>
       </c>
       <c r="O134" s="1" t="s">
         <v>1731</v>
@@ -24670,7 +24674,7 @@
         <v>1617</v>
       </c>
     </row>
-    <row r="135" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="135" spans="1:23">
       <c r="A135" s="1" t="s">
         <v>718</v>
       </c>
@@ -24739,7 +24743,7 @@
         <v>1619</v>
       </c>
     </row>
-    <row r="136" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="136" spans="1:23">
       <c r="A136" s="1" t="s">
         <v>734</v>
       </c>
@@ -24810,7 +24814,7 @@
         <v>1619</v>
       </c>
     </row>
-    <row r="137" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="137" spans="1:23">
       <c r="A137" s="1" t="s">
         <v>734</v>
       </c>
@@ -24879,7 +24883,7 @@
         <v>1617</v>
       </c>
     </row>
-    <row r="138" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="138" spans="1:23">
       <c r="A138" s="1" t="s">
         <v>734</v>
       </c>
@@ -24948,7 +24952,7 @@
         <v>1619</v>
       </c>
     </row>
-    <row r="139" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="139" spans="1:23">
       <c r="A139" s="1" t="s">
         <v>734</v>
       </c>
@@ -25017,7 +25021,7 @@
         <v>1619</v>
       </c>
     </row>
-    <row r="140" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="140" spans="1:23">
       <c r="A140" s="1" t="s">
         <v>752</v>
       </c>
@@ -25086,7 +25090,7 @@
         <v>1619</v>
       </c>
     </row>
-    <row r="141" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="141" spans="1:23">
       <c r="A141" s="1" t="s">
         <v>752</v>
       </c>
@@ -25155,7 +25159,7 @@
         <v>1619</v>
       </c>
     </row>
-    <row r="142" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="142" spans="1:23">
       <c r="A142" s="1" t="s">
         <v>752</v>
       </c>
@@ -25224,7 +25228,7 @@
         <v>1619</v>
       </c>
     </row>
-    <row r="143" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="143" spans="1:23">
       <c r="A143" s="1" t="s">
         <v>752</v>
       </c>
@@ -25293,7 +25297,7 @@
         <v>1617</v>
       </c>
     </row>
-    <row r="144" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="144" spans="1:23">
       <c r="A144" s="1" t="s">
         <v>769</v>
       </c>
@@ -25362,7 +25366,7 @@
         <v>1617</v>
       </c>
     </row>
-    <row r="145" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="145" spans="1:23">
       <c r="A145" s="1" t="s">
         <v>769</v>
       </c>
@@ -25431,7 +25435,7 @@
         <v>1619</v>
       </c>
     </row>
-    <row r="146" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="146" spans="1:23">
       <c r="A146" s="1" t="s">
         <v>769</v>
       </c>
@@ -25500,7 +25504,7 @@
         <v>1617</v>
       </c>
     </row>
-    <row r="147" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="147" spans="1:23">
       <c r="A147" s="1" t="s">
         <v>769</v>
       </c>
@@ -25569,7 +25573,7 @@
         <v>1619</v>
       </c>
     </row>
-    <row r="148" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="148" spans="1:23">
       <c r="A148" s="1" t="s">
         <v>787</v>
       </c>
@@ -25640,7 +25644,7 @@
         <v>1619</v>
       </c>
     </row>
-    <row r="149" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="149" spans="1:23">
       <c r="A149" s="1" t="s">
         <v>787</v>
       </c>
@@ -25681,7 +25685,7 @@
         <v>1642</v>
       </c>
       <c r="N149" s="1">
-        <v>0.29</v>
+        <v>0.28999999999999998</v>
       </c>
       <c r="O149" s="1" t="s">
         <v>1744</v>
@@ -25709,7 +25713,7 @@
         <v>1617</v>
       </c>
     </row>
-    <row r="150" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="150" spans="1:23">
       <c r="A150" s="1" t="s">
         <v>787</v>
       </c>
@@ -25778,7 +25782,7 @@
         <v>1619</v>
       </c>
     </row>
-    <row r="151" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="151" spans="1:23">
       <c r="A151" s="1" t="s">
         <v>787</v>
       </c>
@@ -25819,7 +25823,7 @@
         <v>1630</v>
       </c>
       <c r="N151" s="1">
-        <v>0.29</v>
+        <v>0.28999999999999998</v>
       </c>
       <c r="O151" s="1" t="s">
         <v>1755</v>
@@ -25849,7 +25853,7 @@
         <v>1619</v>
       </c>
     </row>
-    <row r="152" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="152" spans="1:23">
       <c r="A152" s="1" t="s">
         <v>804</v>
       </c>
@@ -25916,7 +25920,7 @@
         <v>1617</v>
       </c>
     </row>
-    <row r="153" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="153" spans="1:23">
       <c r="A153" s="1" t="s">
         <v>804</v>
       </c>
@@ -25985,7 +25989,7 @@
         <v>1619</v>
       </c>
     </row>
-    <row r="154" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="154" spans="1:23">
       <c r="A154" s="1" t="s">
         <v>804</v>
       </c>
@@ -26056,7 +26060,7 @@
         <v>1619</v>
       </c>
     </row>
-    <row r="155" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="155" spans="1:23">
       <c r="A155" s="1" t="s">
         <v>804</v>
       </c>
@@ -26125,7 +26129,7 @@
         <v>1619</v>
       </c>
     </row>
-    <row r="156" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="156" spans="1:23">
       <c r="A156" s="1" t="s">
         <v>821</v>
       </c>
@@ -26194,7 +26198,7 @@
         <v>1619</v>
       </c>
     </row>
-    <row r="157" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="157" spans="1:23">
       <c r="A157" s="1" t="s">
         <v>821</v>
       </c>
@@ -26265,7 +26269,7 @@
         <v>1619</v>
       </c>
     </row>
-    <row r="158" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="158" spans="1:23">
       <c r="A158" s="1" t="s">
         <v>821</v>
       </c>
@@ -26334,7 +26338,7 @@
         <v>1619</v>
       </c>
     </row>
-    <row r="159" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="159" spans="1:23">
       <c r="A159" s="1" t="s">
         <v>821</v>
       </c>
@@ -26401,7 +26405,7 @@
         <v>1617</v>
       </c>
     </row>
-    <row r="160" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="160" spans="1:23">
       <c r="A160" s="1" t="s">
         <v>836</v>
       </c>
@@ -26470,7 +26474,7 @@
         <v>1619</v>
       </c>
     </row>
-    <row r="161" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="161" spans="1:23">
       <c r="A161" s="1" t="s">
         <v>836</v>
       </c>
@@ -26539,7 +26543,7 @@
         <v>1619</v>
       </c>
     </row>
-    <row r="162" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="162" spans="1:23">
       <c r="A162" s="1" t="s">
         <v>836</v>
       </c>
@@ -26578,7 +26582,7 @@
         <v>1630</v>
       </c>
       <c r="N162" s="1">
-        <v>0.57</v>
+        <v>0.56999999999999995</v>
       </c>
       <c r="O162" s="1" t="s">
         <v>1957</v>
@@ -26606,7 +26610,7 @@
         <v>1617</v>
       </c>
     </row>
-    <row r="163" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="163" spans="1:23">
       <c r="A163" s="1" t="s">
         <v>836</v>
       </c>
@@ -26677,7 +26681,7 @@
         <v>1619</v>
       </c>
     </row>
-    <row r="164" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="164" spans="1:23">
       <c r="A164" s="1" t="s">
         <v>853</v>
       </c>
@@ -26748,7 +26752,7 @@
         <v>1617</v>
       </c>
     </row>
-    <row r="165" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="165" spans="1:23">
       <c r="A165" s="1" t="s">
         <v>853</v>
       </c>
@@ -26815,7 +26819,7 @@
         <v>1617</v>
       </c>
     </row>
-    <row r="166" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="166" spans="1:23">
       <c r="A166" s="1" t="s">
         <v>853</v>
       </c>
@@ -26886,7 +26890,7 @@
         <v>1619</v>
       </c>
     </row>
-    <row r="167" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="167" spans="1:23">
       <c r="A167" s="1" t="s">
         <v>853</v>
       </c>
@@ -26955,7 +26959,7 @@
         <v>1617</v>
       </c>
     </row>
-    <row r="168" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="168" spans="1:23">
       <c r="A168" s="1" t="s">
         <v>869</v>
       </c>
@@ -27024,7 +27028,7 @@
         <v>1619</v>
       </c>
     </row>
-    <row r="169" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="169" spans="1:23">
       <c r="A169" s="1" t="s">
         <v>869</v>
       </c>
@@ -27095,7 +27099,7 @@
         <v>1619</v>
       </c>
     </row>
-    <row r="170" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="170" spans="1:23">
       <c r="A170" s="1" t="s">
         <v>869</v>
       </c>
@@ -27164,7 +27168,7 @@
         <v>1617</v>
       </c>
     </row>
-    <row r="171" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="171" spans="1:23">
       <c r="A171" s="1" t="s">
         <v>869</v>
       </c>
@@ -27233,7 +27237,7 @@
         <v>1619</v>
       </c>
     </row>
-    <row r="172" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="172" spans="1:23">
       <c r="A172" s="1" t="s">
         <v>887</v>
       </c>
@@ -27302,7 +27306,7 @@
         <v>1619</v>
       </c>
     </row>
-    <row r="173" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="173" spans="1:23">
       <c r="A173" s="1" t="s">
         <v>887</v>
       </c>
@@ -27371,7 +27375,7 @@
         <v>1617</v>
       </c>
     </row>
-    <row r="174" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="174" spans="1:23">
       <c r="A174" s="1" t="s">
         <v>887</v>
       </c>
@@ -27440,7 +27444,7 @@
         <v>1619</v>
       </c>
     </row>
-    <row r="175" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="175" spans="1:23">
       <c r="A175" s="1" t="s">
         <v>887</v>
       </c>
@@ -27507,7 +27511,7 @@
         <v>1619</v>
       </c>
     </row>
-    <row r="176" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="176" spans="1:23">
       <c r="A176" s="1" t="s">
         <v>904</v>
       </c>
@@ -27576,7 +27580,7 @@
         <v>1617</v>
       </c>
     </row>
-    <row r="177" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="177" spans="1:23">
       <c r="A177" s="1" t="s">
         <v>904</v>
       </c>
@@ -27645,7 +27649,7 @@
         <v>1619</v>
       </c>
     </row>
-    <row r="178" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="178" spans="1:23">
       <c r="A178" s="1" t="s">
         <v>904</v>
       </c>
@@ -27712,7 +27716,7 @@
         <v>1619</v>
       </c>
     </row>
-    <row r="179" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="179" spans="1:23">
       <c r="A179" s="1" t="s">
         <v>904</v>
       </c>
@@ -27783,7 +27787,7 @@
         <v>1619</v>
       </c>
     </row>
-    <row r="180" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="180" spans="1:23">
       <c r="A180" s="1" t="s">
         <v>921</v>
       </c>
@@ -27854,7 +27858,7 @@
         <v>1619</v>
       </c>
     </row>
-    <row r="181" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="181" spans="1:23">
       <c r="A181" s="1" t="s">
         <v>921</v>
       </c>
@@ -27921,7 +27925,7 @@
         <v>1619</v>
       </c>
     </row>
-    <row r="182" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="182" spans="1:23">
       <c r="A182" s="1" t="s">
         <v>921</v>
       </c>
@@ -27992,7 +27996,7 @@
         <v>1619</v>
       </c>
     </row>
-    <row r="183" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="183" spans="1:23">
       <c r="A183" s="1" t="s">
         <v>921</v>
       </c>
@@ -28063,7 +28067,7 @@
         <v>1617</v>
       </c>
     </row>
-    <row r="184" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="184" spans="1:23">
       <c r="A184" s="1" t="s">
         <v>938</v>
       </c>
@@ -28130,7 +28134,7 @@
         <v>1619</v>
       </c>
     </row>
-    <row r="185" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="185" spans="1:23">
       <c r="A185" s="1" t="s">
         <v>938</v>
       </c>
@@ -28201,7 +28205,7 @@
         <v>1619</v>
       </c>
     </row>
-    <row r="186" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="186" spans="1:23">
       <c r="A186" s="1" t="s">
         <v>938</v>
       </c>
@@ -28272,7 +28276,7 @@
         <v>1617</v>
       </c>
     </row>
-    <row r="187" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="187" spans="1:23">
       <c r="A187" s="1" t="s">
         <v>938</v>
       </c>
@@ -28341,7 +28345,7 @@
         <v>1619</v>
       </c>
     </row>
-    <row r="188" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="188" spans="1:23">
       <c r="A188" s="1" t="s">
         <v>954</v>
       </c>
@@ -28410,7 +28414,7 @@
         <v>1619</v>
       </c>
     </row>
-    <row r="189" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="189" spans="1:23">
       <c r="A189" s="1" t="s">
         <v>954</v>
       </c>
@@ -28481,7 +28485,7 @@
         <v>1617</v>
       </c>
     </row>
-    <row r="190" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="190" spans="1:23">
       <c r="A190" s="1" t="s">
         <v>954</v>
       </c>
@@ -28550,7 +28554,7 @@
         <v>1619</v>
       </c>
     </row>
-    <row r="191" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="191" spans="1:23">
       <c r="A191" s="1" t="s">
         <v>954</v>
       </c>
@@ -28617,7 +28621,7 @@
         <v>1617</v>
       </c>
     </row>
-    <row r="192" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="192" spans="1:23">
       <c r="A192" s="1" t="s">
         <v>971</v>
       </c>
@@ -28658,7 +28662,7 @@
         <v>1614</v>
       </c>
       <c r="N192" s="1">
-        <v>0.28</v>
+        <v>0.28000000000000003</v>
       </c>
       <c r="O192" s="1" t="s">
         <v>2011</v>
@@ -28688,7 +28692,7 @@
         <v>1617</v>
       </c>
     </row>
-    <row r="193" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="193" spans="1:23">
       <c r="A193" s="1" t="s">
         <v>971</v>
       </c>
@@ -28757,7 +28761,7 @@
         <v>1619</v>
       </c>
     </row>
-    <row r="194" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="194" spans="1:23">
       <c r="A194" s="1" t="s">
         <v>971</v>
       </c>
@@ -28796,7 +28800,7 @@
         <v>1630</v>
       </c>
       <c r="N194" s="1">
-        <v>0.56</v>
+        <v>0.56000000000000005</v>
       </c>
       <c r="O194" s="1" t="s">
         <v>2008</v>
@@ -28824,7 +28828,7 @@
         <v>1617</v>
       </c>
     </row>
-    <row r="195" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="195" spans="1:23">
       <c r="A195" s="1" t="s">
         <v>971</v>
       </c>
@@ -28893,7 +28897,7 @@
         <v>1619</v>
       </c>
     </row>
-    <row r="196" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="196" spans="1:23">
       <c r="A196" s="1" t="s">
         <v>991</v>
       </c>
@@ -28960,7 +28964,7 @@
         <v>1619</v>
       </c>
     </row>
-    <row r="197" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="197" spans="1:23">
       <c r="A197" s="1" t="s">
         <v>991</v>
       </c>
@@ -29027,7 +29031,7 @@
         <v>1617</v>
       </c>
     </row>
-    <row r="198" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="198" spans="1:23">
       <c r="A198" s="1" t="s">
         <v>991</v>
       </c>
@@ -29096,7 +29100,7 @@
         <v>1619</v>
       </c>
     </row>
-    <row r="199" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="199" spans="1:23">
       <c r="A199" s="1" t="s">
         <v>991</v>
       </c>
@@ -29165,7 +29169,7 @@
         <v>1619</v>
       </c>
     </row>
-    <row r="200" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="200" spans="1:23">
       <c r="A200" s="1" t="s">
         <v>1008</v>
       </c>
@@ -29234,7 +29238,7 @@
         <v>1619</v>
       </c>
     </row>
-    <row r="201" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="201" spans="1:23">
       <c r="A201" s="1" t="s">
         <v>1008</v>
       </c>
@@ -29303,7 +29307,7 @@
         <v>1619</v>
       </c>
     </row>
-    <row r="202" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="202" spans="1:23">
       <c r="A202" s="1" t="s">
         <v>1008</v>
       </c>
@@ -29372,7 +29376,7 @@
         <v>1619</v>
       </c>
     </row>
-    <row r="203" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="203" spans="1:23">
       <c r="A203" s="1" t="s">
         <v>1008</v>
       </c>
@@ -29443,7 +29447,7 @@
         <v>1619</v>
       </c>
     </row>
-    <row r="204" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="204" spans="1:23">
       <c r="A204" s="1" t="s">
         <v>1025</v>
       </c>
@@ -29512,7 +29516,7 @@
         <v>1619</v>
       </c>
     </row>
-    <row r="205" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="205" spans="1:23">
       <c r="A205" s="1" t="s">
         <v>1025</v>
       </c>
@@ -29581,7 +29585,7 @@
         <v>1619</v>
       </c>
     </row>
-    <row r="206" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="206" spans="1:23">
       <c r="A206" s="1" t="s">
         <v>1025</v>
       </c>
@@ -29652,7 +29656,7 @@
         <v>1619</v>
       </c>
     </row>
-    <row r="207" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="207" spans="1:23">
       <c r="A207" s="1" t="s">
         <v>1025</v>
       </c>
@@ -29721,7 +29725,7 @@
         <v>1617</v>
       </c>
     </row>
-    <row r="208" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="208" spans="1:23">
       <c r="A208" s="1" t="s">
         <v>1042</v>
       </c>
@@ -29790,7 +29794,7 @@
         <v>1619</v>
       </c>
     </row>
-    <row r="209" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="209" spans="1:23">
       <c r="A209" s="1" t="s">
         <v>1042</v>
       </c>
@@ -29861,7 +29865,7 @@
         <v>1619</v>
       </c>
     </row>
-    <row r="210" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="210" spans="1:23">
       <c r="A210" s="1" t="s">
         <v>1042</v>
       </c>
@@ -29930,7 +29934,7 @@
         <v>1617</v>
       </c>
     </row>
-    <row r="211" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="211" spans="1:23">
       <c r="A211" s="1" t="s">
         <v>1042</v>
       </c>
@@ -29999,7 +30003,7 @@
         <v>1619</v>
       </c>
     </row>
-    <row r="212" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="212" spans="1:23">
       <c r="A212" s="1" t="s">
         <v>1062</v>
       </c>
@@ -30070,7 +30074,7 @@
         <v>1619</v>
       </c>
     </row>
-    <row r="213" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="213" spans="1:23">
       <c r="A213" s="1" t="s">
         <v>1062</v>
       </c>
@@ -30139,7 +30143,7 @@
         <v>1617</v>
       </c>
     </row>
-    <row r="214" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="214" spans="1:23">
       <c r="A214" s="1" t="s">
         <v>1062</v>
       </c>
@@ -30208,7 +30212,7 @@
         <v>1619</v>
       </c>
     </row>
-    <row r="215" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="215" spans="1:23">
       <c r="A215" s="1" t="s">
         <v>1062</v>
       </c>
@@ -30275,7 +30279,7 @@
         <v>1617</v>
       </c>
     </row>
-    <row r="216" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="216" spans="1:23">
       <c r="A216" s="1" t="s">
         <v>1080</v>
       </c>
@@ -30344,7 +30348,7 @@
         <v>1617</v>
       </c>
     </row>
-    <row r="217" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="217" spans="1:23">
       <c r="A217" s="1" t="s">
         <v>1080</v>
       </c>
@@ -30385,7 +30389,7 @@
         <v>1614</v>
       </c>
       <c r="N217" s="1">
-        <v>0.56</v>
+        <v>0.56000000000000005</v>
       </c>
       <c r="O217" s="1" t="s">
         <v>2033</v>
@@ -30413,7 +30417,7 @@
         <v>1619</v>
       </c>
     </row>
-    <row r="218" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="218" spans="1:23">
       <c r="A218" s="1" t="s">
         <v>1080</v>
       </c>
@@ -30480,7 +30484,7 @@
         <v>1617</v>
       </c>
     </row>
-    <row r="219" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="219" spans="1:23">
       <c r="A219" s="1" t="s">
         <v>1080</v>
       </c>
@@ -30551,7 +30555,7 @@
         <v>1619</v>
       </c>
     </row>
-    <row r="220" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="220" spans="1:23">
       <c r="A220" s="1" t="s">
         <v>1099</v>
       </c>
@@ -30620,7 +30624,7 @@
         <v>1619</v>
       </c>
     </row>
-    <row r="221" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="221" spans="1:23">
       <c r="A221" s="1" t="s">
         <v>1099</v>
       </c>
@@ -30687,7 +30691,7 @@
         <v>1617</v>
       </c>
     </row>
-    <row r="222" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="222" spans="1:23">
       <c r="A222" s="1" t="s">
         <v>1099</v>
       </c>
@@ -30758,7 +30762,7 @@
         <v>1619</v>
       </c>
     </row>
-    <row r="223" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="223" spans="1:23">
       <c r="A223" s="1" t="s">
         <v>1099</v>
       </c>
@@ -30827,7 +30831,7 @@
         <v>1619</v>
       </c>
     </row>
-    <row r="224" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="224" spans="1:23">
       <c r="A224" s="1" t="s">
         <v>1116</v>
       </c>
@@ -30894,7 +30898,7 @@
         <v>1617</v>
       </c>
     </row>
-    <row r="225" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="225" spans="1:23">
       <c r="A225" s="1" t="s">
         <v>1116</v>
       </c>
@@ -30965,7 +30969,7 @@
         <v>1619</v>
       </c>
     </row>
-    <row r="226" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="226" spans="1:23">
       <c r="A226" s="1" t="s">
         <v>1116</v>
       </c>
@@ -31034,7 +31038,7 @@
         <v>1619</v>
       </c>
     </row>
-    <row r="227" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="227" spans="1:23">
       <c r="A227" s="1" t="s">
         <v>1116</v>
       </c>
@@ -31103,7 +31107,7 @@
         <v>1617</v>
       </c>
     </row>
-    <row r="228" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="228" spans="1:23">
       <c r="A228" s="1" t="s">
         <v>1135</v>
       </c>
@@ -31144,7 +31148,7 @@
         <v>1614</v>
       </c>
       <c r="N228" s="1">
-        <v>0.57</v>
+        <v>0.56999999999999995</v>
       </c>
       <c r="O228" s="1" t="s">
         <v>2038</v>
@@ -31174,7 +31178,7 @@
         <v>1619</v>
       </c>
     </row>
-    <row r="229" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="229" spans="1:23">
       <c r="A229" s="1" t="s">
         <v>1135</v>
       </c>
@@ -31243,7 +31247,7 @@
         <v>1619</v>
       </c>
     </row>
-    <row r="230" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="230" spans="1:23">
       <c r="A230" s="1" t="s">
         <v>1135</v>
       </c>
@@ -31312,7 +31316,7 @@
         <v>1617</v>
       </c>
     </row>
-    <row r="231" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="231" spans="1:23">
       <c r="A231" s="1" t="s">
         <v>1135</v>
       </c>
@@ -31383,7 +31387,7 @@
         <v>1619</v>
       </c>
     </row>
-    <row r="232" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="232" spans="1:23">
       <c r="A232" s="1" t="s">
         <v>1155</v>
       </c>
@@ -31452,7 +31456,7 @@
         <v>1619</v>
       </c>
     </row>
-    <row r="233" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="233" spans="1:23">
       <c r="A233" s="1" t="s">
         <v>1155</v>
       </c>
@@ -31521,7 +31525,7 @@
         <v>1617</v>
       </c>
     </row>
-    <row r="234" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="234" spans="1:23">
       <c r="A234" s="1" t="s">
         <v>1155</v>
       </c>
@@ -31592,7 +31596,7 @@
         <v>1619</v>
       </c>
     </row>
-    <row r="235" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="235" spans="1:23">
       <c r="A235" s="1" t="s">
         <v>1155</v>
       </c>
@@ -31661,7 +31665,7 @@
         <v>1619</v>
       </c>
     </row>
-    <row r="236" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="236" spans="1:23">
       <c r="A236" s="1" t="s">
         <v>1174</v>
       </c>
@@ -31730,7 +31734,7 @@
         <v>1617</v>
       </c>
     </row>
-    <row r="237" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="237" spans="1:23">
       <c r="A237" s="1" t="s">
         <v>1174</v>
       </c>
@@ -31801,7 +31805,7 @@
         <v>1619</v>
       </c>
     </row>
-    <row r="238" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="238" spans="1:23">
       <c r="A238" s="1" t="s">
         <v>1174</v>
       </c>
@@ -31870,7 +31874,7 @@
         <v>1619</v>
       </c>
     </row>
-    <row r="239" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="239" spans="1:23">
       <c r="A239" s="1" t="s">
         <v>1174</v>
       </c>
@@ -31937,7 +31941,7 @@
         <v>1617</v>
       </c>
     </row>
-    <row r="240" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="240" spans="1:23">
       <c r="A240" s="1" t="s">
         <v>1193</v>
       </c>
@@ -32008,7 +32012,7 @@
         <v>1619</v>
       </c>
     </row>
-    <row r="241" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="241" spans="1:23">
       <c r="A241" s="1" t="s">
         <v>1193</v>
       </c>
@@ -32077,7 +32081,7 @@
         <v>1619</v>
       </c>
     </row>
-    <row r="242" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="242" spans="1:23">
       <c r="A242" s="1" t="s">
         <v>1193</v>
       </c>
@@ -32144,7 +32148,7 @@
         <v>1617</v>
       </c>
     </row>
-    <row r="243" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="243" spans="1:23">
       <c r="A243" s="1" t="s">
         <v>1193</v>
       </c>
@@ -32185,7 +32189,7 @@
         <v>1630</v>
       </c>
       <c r="N243" s="1">
-        <v>0.56</v>
+        <v>0.56000000000000005</v>
       </c>
       <c r="O243" s="1" t="s">
         <v>2057</v>
@@ -32215,7 +32219,7 @@
         <v>1619</v>
       </c>
     </row>
-    <row r="244" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="244" spans="1:23">
       <c r="A244" s="1" t="s">
         <v>1212</v>
       </c>
@@ -32284,7 +32288,7 @@
         <v>1619</v>
       </c>
     </row>
-    <row r="245" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="245" spans="1:23">
       <c r="A245" s="1" t="s">
         <v>1212</v>
       </c>
@@ -32351,7 +32355,7 @@
         <v>1617</v>
       </c>
     </row>
-    <row r="246" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="246" spans="1:23">
       <c r="A246" s="1" t="s">
         <v>1212</v>
       </c>
@@ -32422,7 +32426,7 @@
         <v>1619</v>
       </c>
     </row>
-    <row r="247" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="247" spans="1:23">
       <c r="A247" s="1" t="s">
         <v>1212</v>
       </c>
@@ -32491,7 +32495,7 @@
         <v>1619</v>
       </c>
     </row>
-    <row r="248" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="248" spans="1:23">
       <c r="A248" s="1" t="s">
         <v>1228</v>
       </c>
@@ -32558,7 +32562,7 @@
         <v>1617</v>
       </c>
     </row>
-    <row r="249" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="249" spans="1:23">
       <c r="A249" s="1" t="s">
         <v>1228</v>
       </c>
@@ -32629,7 +32633,7 @@
         <v>1619</v>
       </c>
     </row>
-    <row r="250" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="250" spans="1:23">
       <c r="A250" s="1" t="s">
         <v>1228</v>
       </c>
@@ -32698,7 +32702,7 @@
         <v>1619</v>
       </c>
     </row>
-    <row r="251" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="251" spans="1:23">
       <c r="A251" s="1" t="s">
         <v>1228</v>
       </c>
@@ -32739,7 +32743,7 @@
         <v>1614</v>
       </c>
       <c r="N251" s="1">
-        <v>0.58</v>
+        <v>0.57999999999999996</v>
       </c>
       <c r="O251" s="1" t="s">
         <v>1891</v>
@@ -32767,7 +32771,7 @@
         <v>1617</v>
       </c>
     </row>
-    <row r="252" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="252" spans="1:23">
       <c r="A252" s="1" t="s">
         <v>1247</v>
       </c>
@@ -32838,7 +32842,7 @@
         <v>1619</v>
       </c>
     </row>
-    <row r="253" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="253" spans="1:23">
       <c r="A253" s="1" t="s">
         <v>1247</v>
       </c>
@@ -32907,7 +32911,7 @@
         <v>1619</v>
       </c>
     </row>
-    <row r="254" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="254" spans="1:23">
       <c r="A254" s="1" t="s">
         <v>1247</v>
       </c>
@@ -32976,7 +32980,7 @@
         <v>1617</v>
       </c>
     </row>
-    <row r="255" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="255" spans="1:23">
       <c r="A255" s="1" t="s">
         <v>1247</v>
       </c>
@@ -33045,7 +33049,7 @@
         <v>1619</v>
       </c>
     </row>
-    <row r="256" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="256" spans="1:23">
       <c r="A256" s="1" t="s">
         <v>1267</v>
       </c>
@@ -33114,7 +33118,7 @@
         <v>1619</v>
       </c>
     </row>
-    <row r="257" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="257" spans="1:23">
       <c r="A257" s="1" t="s">
         <v>1267</v>
       </c>
@@ -33183,7 +33187,7 @@
         <v>1617</v>
       </c>
     </row>
-    <row r="258" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="258" spans="1:23">
       <c r="A258" s="1" t="s">
         <v>1267</v>
       </c>
@@ -33252,7 +33256,7 @@
         <v>1619</v>
       </c>
     </row>
-    <row r="259" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="259" spans="1:23">
       <c r="A259" s="1" t="s">
         <v>1267</v>
       </c>
@@ -33323,7 +33327,7 @@
         <v>1619</v>
       </c>
     </row>
-    <row r="260" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="260" spans="1:23">
       <c r="A260" s="1" t="s">
         <v>1284</v>
       </c>
@@ -33392,7 +33396,7 @@
         <v>1617</v>
       </c>
     </row>
-    <row r="261" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="261" spans="1:23">
       <c r="A261" s="1" t="s">
         <v>1284</v>
       </c>
@@ -33461,7 +33465,7 @@
         <v>1619</v>
       </c>
     </row>
-    <row r="262" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="262" spans="1:23">
       <c r="A262" s="1" t="s">
         <v>1284</v>
       </c>
@@ -33532,7 +33536,7 @@
         <v>1619</v>
       </c>
     </row>
-    <row r="263" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="263" spans="1:23">
       <c r="A263" s="1" t="s">
         <v>1284</v>
       </c>
@@ -33601,7 +33605,7 @@
         <v>1619</v>
       </c>
     </row>
-    <row r="264" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="264" spans="1:23">
       <c r="A264" s="1" t="s">
         <v>1302</v>
       </c>
@@ -33670,7 +33674,7 @@
         <v>1619</v>
       </c>
     </row>
-    <row r="265" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="265" spans="1:23">
       <c r="A265" s="1" t="s">
         <v>1302</v>
       </c>
@@ -33741,7 +33745,7 @@
         <v>1619</v>
       </c>
     </row>
-    <row r="266" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="266" spans="1:23">
       <c r="A266" s="1" t="s">
         <v>1302</v>
       </c>
@@ -33810,7 +33814,7 @@
         <v>1619</v>
       </c>
     </row>
-    <row r="267" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="267" spans="1:23">
       <c r="A267" s="1" t="s">
         <v>1302</v>
       </c>
@@ -33877,7 +33881,7 @@
         <v>1617</v>
       </c>
     </row>
-    <row r="268" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="268" spans="1:23">
       <c r="A268" s="1" t="s">
         <v>1319</v>
       </c>
@@ -33948,7 +33952,7 @@
         <v>1619</v>
       </c>
     </row>
-    <row r="269" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="269" spans="1:23">
       <c r="A269" s="1" t="s">
         <v>1319</v>
       </c>
@@ -34017,7 +34021,7 @@
         <v>1619</v>
       </c>
     </row>
-    <row r="270" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="270" spans="1:23">
       <c r="A270" s="1" t="s">
         <v>1319</v>
       </c>
@@ -34084,7 +34088,7 @@
         <v>1617</v>
       </c>
     </row>
-    <row r="271" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="271" spans="1:23">
       <c r="A271" s="1" t="s">
         <v>1319</v>
       </c>
@@ -34153,7 +34157,7 @@
         <v>1619</v>
       </c>
     </row>
-    <row r="272" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="272" spans="1:23">
       <c r="A272" s="1" t="s">
         <v>1338</v>
       </c>
@@ -34222,7 +34226,7 @@
         <v>1619</v>
       </c>
     </row>
-    <row r="273" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="273" spans="1:23">
       <c r="A273" s="1" t="s">
         <v>1338</v>
       </c>
@@ -34289,7 +34293,7 @@
         <v>1617</v>
       </c>
     </row>
-    <row r="274" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="274" spans="1:23">
       <c r="A274" s="1" t="s">
         <v>1338</v>
       </c>
@@ -34358,7 +34362,7 @@
         <v>1619</v>
       </c>
     </row>
-    <row r="275" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="275" spans="1:23">
       <c r="A275" s="1" t="s">
         <v>1338</v>
       </c>
@@ -34427,7 +34431,7 @@
         <v>1619</v>
       </c>
     </row>
-    <row r="276" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="276" spans="1:23">
       <c r="A276" s="1" t="s">
         <v>1358</v>
       </c>
@@ -34494,7 +34498,7 @@
         <v>1617</v>
       </c>
     </row>
-    <row r="277" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="277" spans="1:23">
       <c r="A277" s="1" t="s">
         <v>1358</v>
       </c>
@@ -34563,7 +34567,7 @@
         <v>1619</v>
       </c>
     </row>
-    <row r="278" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="278" spans="1:23">
       <c r="A278" s="1" t="s">
         <v>1358</v>
       </c>
@@ -34632,7 +34636,7 @@
         <v>1619</v>
       </c>
     </row>
-    <row r="279" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="279" spans="1:23">
       <c r="A279" s="1" t="s">
         <v>1358</v>
       </c>
@@ -34701,7 +34705,7 @@
         <v>1617</v>
       </c>
     </row>
-    <row r="280" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="280" spans="1:23">
       <c r="A280" s="1" t="s">
         <v>1375</v>
       </c>
@@ -34740,7 +34744,7 @@
         <v>1614</v>
       </c>
       <c r="N280" s="1">
-        <v>0.14</v>
+        <v>0.14000000000000001</v>
       </c>
       <c r="O280" s="1" t="s">
         <v>2081</v>
@@ -34770,7 +34774,7 @@
         <v>1619</v>
       </c>
     </row>
-    <row r="281" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="281" spans="1:23">
       <c r="A281" s="1" t="s">
         <v>1375</v>
       </c>
@@ -34839,7 +34843,7 @@
         <v>1619</v>
       </c>
     </row>
-    <row r="282" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="282" spans="1:23">
       <c r="A282" s="1" t="s">
         <v>1375</v>
       </c>
@@ -34880,7 +34884,7 @@
         <v>1630</v>
       </c>
       <c r="N282" s="1">
-        <v>0.58</v>
+        <v>0.57999999999999996</v>
       </c>
       <c r="O282" s="1" t="s">
         <v>2086</v>
@@ -34908,7 +34912,7 @@
         <v>1617</v>
       </c>
     </row>
-    <row r="283" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="283" spans="1:23">
       <c r="A283" s="1" t="s">
         <v>1375</v>
       </c>
@@ -34947,7 +34951,7 @@
         <v>1630</v>
       </c>
       <c r="N283" s="1">
-        <v>0.14</v>
+        <v>0.14000000000000001</v>
       </c>
       <c r="O283" s="1" t="s">
         <v>2089</v>
@@ -34975,7 +34979,7 @@
         <v>1619</v>
       </c>
     </row>
-    <row r="284" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="284" spans="1:23">
       <c r="A284" s="1" t="s">
         <v>1392</v>
       </c>
@@ -35044,7 +35048,7 @@
         <v>1619</v>
       </c>
     </row>
-    <row r="285" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="285" spans="1:23">
       <c r="A285" s="1" t="s">
         <v>1392</v>
       </c>
@@ -35085,7 +35089,7 @@
         <v>1630</v>
       </c>
       <c r="N285" s="1">
-        <v>0.56</v>
+        <v>0.56000000000000005</v>
       </c>
       <c r="O285" s="1" t="s">
         <v>2086</v>
@@ -35113,7 +35117,7 @@
         <v>1617</v>
       </c>
     </row>
-    <row r="286" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="286" spans="1:23">
       <c r="A286" s="1" t="s">
         <v>1392</v>
       </c>
@@ -35180,7 +35184,7 @@
         <v>1619</v>
       </c>
     </row>
-    <row r="287" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="287" spans="1:23">
       <c r="A287" s="1" t="s">
         <v>1392</v>
       </c>
@@ -35251,7 +35255,7 @@
         <v>1617</v>
       </c>
     </row>
-    <row r="288" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="288" spans="1:23">
       <c r="A288" s="1" t="s">
         <v>1409</v>
       </c>
@@ -35292,7 +35296,7 @@
         <v>1630</v>
       </c>
       <c r="N288" s="1">
-        <v>0.29</v>
+        <v>0.28999999999999998</v>
       </c>
       <c r="O288" s="1" t="s">
         <v>2086</v>
@@ -35320,7 +35324,7 @@
         <v>1617</v>
       </c>
     </row>
-    <row r="289" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="289" spans="1:23">
       <c r="A289" s="1" t="s">
         <v>1409</v>
       </c>
@@ -35387,7 +35391,7 @@
         <v>1619</v>
       </c>
     </row>
-    <row r="290" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="290" spans="1:23">
       <c r="A290" s="1" t="s">
         <v>1409</v>
       </c>
@@ -35458,7 +35462,7 @@
         <v>1617</v>
       </c>
     </row>
-    <row r="291" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="291" spans="1:23">
       <c r="A291" s="1" t="s">
         <v>1409</v>
       </c>
@@ -35527,7 +35531,7 @@
         <v>1619</v>
       </c>
     </row>
-    <row r="292" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="292" spans="1:23">
       <c r="A292" s="1" t="s">
         <v>1427</v>
       </c>
@@ -35594,7 +35598,7 @@
         <v>1619</v>
       </c>
     </row>
-    <row r="293" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="293" spans="1:23">
       <c r="A293" s="1" t="s">
         <v>1427</v>
       </c>
@@ -35665,7 +35669,7 @@
         <v>1617</v>
       </c>
     </row>
-    <row r="294" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="294" spans="1:23">
       <c r="A294" s="1" t="s">
         <v>1427</v>
       </c>
@@ -35734,7 +35738,7 @@
         <v>1619</v>
       </c>
     </row>
-    <row r="295" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="295" spans="1:23">
       <c r="A295" s="1" t="s">
         <v>1427</v>
       </c>
@@ -35801,7 +35805,7 @@
         <v>1619</v>
       </c>
     </row>
-    <row r="296" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="296" spans="1:23">
       <c r="A296" s="1" t="s">
         <v>1442</v>
       </c>
@@ -35872,7 +35876,7 @@
         <v>1617</v>
       </c>
     </row>
-    <row r="297" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="297" spans="1:23">
       <c r="A297" s="1" t="s">
         <v>1442</v>
       </c>
@@ -35941,7 +35945,7 @@
         <v>1619</v>
       </c>
     </row>
-    <row r="298" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="298" spans="1:23">
       <c r="A298" s="1" t="s">
         <v>1442</v>
       </c>
@@ -36008,7 +36012,7 @@
         <v>1619</v>
       </c>
     </row>
-    <row r="299" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="299" spans="1:23">
       <c r="A299" s="1" t="s">
         <v>1442</v>
       </c>
@@ -36079,7 +36083,7 @@
         <v>1619</v>
       </c>
     </row>
-    <row r="300" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="300" spans="1:23">
       <c r="A300" s="1" t="s">
         <v>1457</v>
       </c>
@@ -36120,7 +36124,7 @@
         <v>1630</v>
       </c>
       <c r="N300" s="1">
-        <v>0.55</v>
+        <v>0.55000000000000004</v>
       </c>
       <c r="O300" s="1" t="s">
         <v>2095</v>
@@ -36148,7 +36152,7 @@
         <v>1619</v>
       </c>
     </row>
-    <row r="301" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="301" spans="1:23">
       <c r="A301" s="1" t="s">
         <v>1457</v>
       </c>
@@ -36215,7 +36219,7 @@
         <v>1619</v>
       </c>
     </row>
-    <row r="302" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="302" spans="1:23">
       <c r="A302" s="1" t="s">
         <v>1457</v>
       </c>
@@ -36286,7 +36290,7 @@
         <v>1619</v>
       </c>
     </row>
-    <row r="303" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="303" spans="1:23">
       <c r="A303" s="1" t="s">
         <v>1457</v>
       </c>
@@ -36355,7 +36359,7 @@
         <v>1619</v>
       </c>
     </row>
-    <row r="304" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="304" spans="1:23">
       <c r="A304" s="1" t="s">
         <v>1474</v>
       </c>
@@ -36422,7 +36426,7 @@
         <v>1619</v>
       </c>
     </row>
-    <row r="305" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="305" spans="1:23">
       <c r="A305" s="1" t="s">
         <v>1474</v>
       </c>
@@ -36493,7 +36497,7 @@
         <v>1619</v>
       </c>
     </row>
-    <row r="306" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="306" spans="1:23">
       <c r="A306" s="1" t="s">
         <v>1474</v>
       </c>
@@ -36562,7 +36566,7 @@
         <v>1619</v>
       </c>
     </row>
-    <row r="307" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="307" spans="1:23">
       <c r="A307" s="1" t="s">
         <v>1474</v>
       </c>
@@ -36629,7 +36633,7 @@
         <v>1619</v>
       </c>
     </row>
-    <row r="308" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="308" spans="1:23">
       <c r="A308" s="1" t="s">
         <v>1492</v>
       </c>
@@ -36670,7 +36674,7 @@
         <v>1642</v>
       </c>
       <c r="N308" s="1">
-        <v>0.56</v>
+        <v>0.56000000000000005</v>
       </c>
       <c r="O308" s="1" t="s">
         <v>2102</v>
@@ -36700,7 +36704,7 @@
         <v>1619</v>
       </c>
     </row>
-    <row r="309" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="309" spans="1:23">
       <c r="A309" s="1" t="s">
         <v>1492</v>
       </c>
@@ -36769,7 +36773,7 @@
         <v>1619</v>
       </c>
     </row>
-    <row r="310" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="310" spans="1:23">
       <c r="A310" s="1" t="s">
         <v>1492</v>
       </c>
@@ -36836,7 +36840,7 @@
         <v>1619</v>
       </c>
     </row>
-    <row r="311" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="311" spans="1:23">
       <c r="A311" s="1" t="s">
         <v>1492</v>
       </c>
@@ -36905,7 +36909,7 @@
         <v>1617</v>
       </c>
     </row>
-    <row r="312" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="312" spans="1:23">
       <c r="A312" s="1" t="s">
         <v>1508</v>
       </c>
@@ -36974,7 +36978,7 @@
         <v>1619</v>
       </c>
     </row>
-    <row r="313" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="313" spans="1:23">
       <c r="A313" s="1" t="s">
         <v>1508</v>
       </c>
@@ -37041,7 +37045,7 @@
         <v>1619</v>
       </c>
     </row>
-    <row r="314" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="314" spans="1:23">
       <c r="A314" s="1" t="s">
         <v>1508</v>
       </c>
@@ -37110,7 +37114,7 @@
         <v>1617</v>
       </c>
     </row>
-    <row r="315" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="315" spans="1:23">
       <c r="A315" s="1" t="s">
         <v>1508</v>
       </c>
@@ -37179,7 +37183,7 @@
         <v>1619</v>
       </c>
     </row>
-    <row r="316" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="316" spans="1:23">
       <c r="A316" s="1" t="s">
         <v>1523</v>
       </c>
@@ -37246,7 +37250,7 @@
         <v>1619</v>
       </c>
     </row>
-    <row r="317" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="317" spans="1:23">
       <c r="A317" s="1" t="s">
         <v>1523</v>
       </c>
@@ -37315,7 +37319,7 @@
         <v>1617</v>
       </c>
     </row>
-    <row r="318" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="318" spans="1:23">
       <c r="A318" s="1" t="s">
         <v>1523</v>
       </c>
@@ -37384,7 +37388,7 @@
         <v>1619</v>
       </c>
     </row>
-    <row r="319" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="319" spans="1:23">
       <c r="A319" s="1" t="s">
         <v>1523</v>
       </c>
@@ -37453,7 +37457,7 @@
         <v>1617</v>
       </c>
     </row>
-    <row r="320" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="320" spans="1:23">
       <c r="A320" s="1" t="s">
         <v>1538</v>
       </c>
@@ -37522,7 +37526,7 @@
         <v>1617</v>
       </c>
     </row>
-    <row r="321" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="321" spans="1:23">
       <c r="A321" s="1" t="s">
         <v>1538</v>
       </c>
@@ -37563,7 +37567,7 @@
         <v>1642</v>
       </c>
       <c r="N321" s="1">
-        <v>0.58</v>
+        <v>0.57999999999999996</v>
       </c>
       <c r="O321" s="1" t="s">
         <v>2115</v>
@@ -37591,7 +37595,7 @@
         <v>1619</v>
       </c>
     </row>
-    <row r="322" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="322" spans="1:23">
       <c r="A322" s="1" t="s">
         <v>1538</v>
       </c>
@@ -37660,7 +37664,7 @@
         <v>1617</v>
       </c>
     </row>
-    <row r="323" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="323" spans="1:23">
       <c r="A323" s="1" t="s">
         <v>1538</v>
       </c>
@@ -37731,7 +37735,7 @@
         <v>1619</v>
       </c>
     </row>
-    <row r="324" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="324" spans="1:23">
       <c r="A324" s="1" t="s">
         <v>1557</v>
       </c>
@@ -37800,7 +37804,7 @@
         <v>1619</v>
       </c>
     </row>
-    <row r="325" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="325" spans="1:23">
       <c r="A325" s="1" t="s">
         <v>1557</v>
       </c>
@@ -37869,7 +37873,7 @@
         <v>1617</v>
       </c>
     </row>
-    <row r="326" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="326" spans="1:23">
       <c r="A326" s="1" t="s">
         <v>1557</v>
       </c>
@@ -37940,7 +37944,7 @@
         <v>1619</v>
       </c>
     </row>
-    <row r="327" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="327" spans="1:23">
       <c r="A327" s="1" t="s">
         <v>1557</v>
       </c>
@@ -37979,7 +37983,7 @@
         <v>1630</v>
       </c>
       <c r="N327" s="1">
-        <v>0.29</v>
+        <v>0.28999999999999998</v>
       </c>
       <c r="O327" s="1" t="s">
         <v>2125</v>
@@ -38007,7 +38011,7 @@
         <v>1619</v>
       </c>
     </row>
-    <row r="328" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="328" spans="1:23">
       <c r="A328" s="1" t="s">
         <v>1574</v>
       </c>
@@ -38076,7 +38080,7 @@
         <v>1617</v>
       </c>
     </row>
-    <row r="329" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="329" spans="1:23">
       <c r="A329" s="1" t="s">
         <v>1574</v>
       </c>
@@ -38147,7 +38151,7 @@
         <v>1619</v>
       </c>
     </row>
-    <row r="330" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="330" spans="1:23">
       <c r="A330" s="1" t="s">
         <v>1574</v>
       </c>
@@ -38214,7 +38218,7 @@
         <v>1619</v>
       </c>
     </row>
-    <row r="331" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="331" spans="1:23">
       <c r="A331" s="1" t="s">
         <v>1574</v>
       </c>
@@ -38284,26 +38288,26 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:W1"/>
+  <autoFilter ref="A1:W1" xr:uid="{00000000-0009-0000-0000-000001000000}"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1:E83"/>
-  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+  <sheetFormatPr defaultRowHeight="14.4"/>
   <cols>
-    <col min="1" max="1" width="19.285714285714285" customWidth="1"/>
-    <col min="2" max="2" width="16.285714285714285" customWidth="1"/>
+    <col min="1" max="1" width="19.33203125" customWidth="1"/>
+    <col min="2" max="2" width="16.33203125" customWidth="1"/>
     <col min="3" max="3" width="33" customWidth="1"/>
     <col min="4" max="4" width="23" customWidth="1"/>
     <col min="5" max="5" width="29" customWidth="1"/>
-    <col min="6" max="24" width="13.571428571428571" customWidth="1"/>
+    <col min="6" max="24" width="13.5546875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:5">
       <c r="A1" s="1" t="s">
         <v>2129</v>
       </c>
@@ -38320,7 +38324,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:5">
       <c r="A2" s="1" t="s">
         <v>34</v>
       </c>
@@ -38337,7 +38341,7 @@
         <v>0.15</v>
       </c>
     </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:5">
       <c r="A3" s="1" t="s">
         <v>58</v>
       </c>
@@ -38354,7 +38358,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:5">
       <c r="A4" s="1" t="s">
         <v>84</v>
       </c>
@@ -38371,7 +38375,7 @@
         <v>0.15</v>
       </c>
     </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:5">
       <c r="A5" s="1" t="s">
         <v>104</v>
       </c>
@@ -38388,7 +38392,7 @@
         <v>119</v>
       </c>
     </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:5">
       <c r="A6" s="1" t="s">
         <v>129</v>
       </c>
@@ -38405,7 +38409,7 @@
         <v>142</v>
       </c>
     </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:5">
       <c r="A7" s="1" t="s">
         <v>150</v>
       </c>
@@ -38422,7 +38426,7 @@
         <v>0.15</v>
       </c>
     </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:5">
       <c r="A8" s="1" t="s">
         <v>175</v>
       </c>
@@ -38439,7 +38443,7 @@
         <v>189</v>
       </c>
     </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:5">
       <c r="A9" s="1" t="s">
         <v>196</v>
       </c>
@@ -38456,7 +38460,7 @@
         <v>211</v>
       </c>
     </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:5">
       <c r="A10" s="1" t="s">
         <v>219</v>
       </c>
@@ -38473,7 +38477,7 @@
         <v>232</v>
       </c>
     </row>
-    <row r="11" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:5">
       <c r="A11" s="1" t="s">
         <v>240</v>
       </c>
@@ -38490,7 +38494,7 @@
         <v>254</v>
       </c>
     </row>
-    <row r="12" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:5">
       <c r="A12" s="1" t="s">
         <v>262</v>
       </c>
@@ -38507,7 +38511,7 @@
         <v>0.15</v>
       </c>
     </row>
-    <row r="13" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:5">
       <c r="A13" s="1" t="s">
         <v>282</v>
       </c>
@@ -38524,7 +38528,7 @@
         <v>297</v>
       </c>
     </row>
-    <row r="14" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:5">
       <c r="A14" s="1" t="s">
         <v>306</v>
       </c>
@@ -38541,7 +38545,7 @@
         <v>0.15</v>
       </c>
     </row>
-    <row r="15" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:5">
       <c r="A15" s="1" t="s">
         <v>326</v>
       </c>
@@ -38558,7 +38562,7 @@
         <v>341</v>
       </c>
     </row>
-    <row r="16" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:5">
       <c r="A16" s="1" t="s">
         <v>350</v>
       </c>
@@ -38575,7 +38579,7 @@
         <v>363</v>
       </c>
     </row>
-    <row r="17" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:5">
       <c r="A17" s="1" t="s">
         <v>371</v>
       </c>
@@ -38592,7 +38596,7 @@
         <v>386</v>
       </c>
     </row>
-    <row r="18" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:5">
       <c r="A18" s="1" t="s">
         <v>395</v>
       </c>
@@ -38609,7 +38613,7 @@
         <v>410</v>
       </c>
     </row>
-    <row r="19" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:5">
       <c r="A19" s="1" t="s">
         <v>418</v>
       </c>
@@ -38626,7 +38630,7 @@
         <v>433</v>
       </c>
     </row>
-    <row r="20" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:5">
       <c r="A20" s="1" t="s">
         <v>442</v>
       </c>
@@ -38643,7 +38647,7 @@
         <v>297</v>
       </c>
     </row>
-    <row r="21" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:5">
       <c r="A21" s="1" t="s">
         <v>463</v>
       </c>
@@ -38660,7 +38664,7 @@
         <v>477</v>
       </c>
     </row>
-    <row r="22" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:5">
       <c r="A22" s="1" t="s">
         <v>485</v>
       </c>
@@ -38677,7 +38681,7 @@
         <v>232</v>
       </c>
     </row>
-    <row r="23" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:5">
       <c r="A23" s="1" t="s">
         <v>505</v>
       </c>
@@ -38694,7 +38698,7 @@
         <v>0.15</v>
       </c>
     </row>
-    <row r="24" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:5">
       <c r="A24" s="1" t="s">
         <v>527</v>
       </c>
@@ -38711,7 +38715,7 @@
         <v>539</v>
       </c>
     </row>
-    <row r="25" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:5">
       <c r="A25" s="1" t="s">
         <v>548</v>
       </c>
@@ -38728,7 +38732,7 @@
         <v>0.15</v>
       </c>
     </row>
-    <row r="26" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:5">
       <c r="A26" s="1" t="s">
         <v>568</v>
       </c>
@@ -38742,10 +38746,10 @@
         <v>4</v>
       </c>
       <c r="E26" s="2">
-        <v>0.14</v>
-      </c>
-    </row>
-    <row r="27" spans="1:5" x14ac:dyDescent="0.25">
+        <v>0.14000000000000001</v>
+      </c>
+    </row>
+    <row r="27" spans="1:5">
       <c r="A27" s="1" t="s">
         <v>585</v>
       </c>
@@ -38762,7 +38766,7 @@
         <v>0.16</v>
       </c>
     </row>
-    <row r="28" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:5">
       <c r="A28" s="1" t="s">
         <v>605</v>
       </c>
@@ -38779,7 +38783,7 @@
         <v>0.11</v>
       </c>
     </row>
-    <row r="29" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:5">
       <c r="A29" s="1" t="s">
         <v>623</v>
       </c>
@@ -38796,7 +38800,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="30" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:5">
       <c r="A30" s="1" t="s">
         <v>642</v>
       </c>
@@ -38813,7 +38817,7 @@
         <v>0.18</v>
       </c>
     </row>
-    <row r="31" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:5">
       <c r="A31" s="1" t="s">
         <v>660</v>
       </c>
@@ -38830,7 +38834,7 @@
         <v>0.12</v>
       </c>
     </row>
-    <row r="32" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:5">
       <c r="A32" s="1" t="s">
         <v>679</v>
       </c>
@@ -38847,7 +38851,7 @@
         <v>0.19</v>
       </c>
     </row>
-    <row r="33" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:5">
       <c r="A33" s="1" t="s">
         <v>699</v>
       </c>
@@ -38864,7 +38868,7 @@
         <v>0.1</v>
       </c>
     </row>
-    <row r="34" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:5">
       <c r="A34" s="1" t="s">
         <v>718</v>
       </c>
@@ -38881,7 +38885,7 @@
         <v>0.17</v>
       </c>
     </row>
-    <row r="35" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:5">
       <c r="A35" s="1" t="s">
         <v>734</v>
       </c>
@@ -38898,7 +38902,7 @@
         <v>0.13</v>
       </c>
     </row>
-    <row r="36" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:5">
       <c r="A36" s="1" t="s">
         <v>752</v>
       </c>
@@ -38915,7 +38919,7 @@
         <v>762</v>
       </c>
     </row>
-    <row r="37" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:5">
       <c r="A37" s="1" t="s">
         <v>769</v>
       </c>
@@ -38932,7 +38936,7 @@
         <v>433</v>
       </c>
     </row>
-    <row r="38" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:5">
       <c r="A38" s="1" t="s">
         <v>787</v>
       </c>
@@ -38949,7 +38953,7 @@
         <v>297</v>
       </c>
     </row>
-    <row r="39" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:5">
       <c r="A39" s="1" t="s">
         <v>804</v>
       </c>
@@ -38966,7 +38970,7 @@
         <v>477</v>
       </c>
     </row>
-    <row r="40" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:5">
       <c r="A40" s="1" t="s">
         <v>821</v>
       </c>
@@ -38983,7 +38987,7 @@
         <v>386</v>
       </c>
     </row>
-    <row r="41" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:5">
       <c r="A41" s="1" t="s">
         <v>836</v>
       </c>
@@ -39000,7 +39004,7 @@
         <v>341</v>
       </c>
     </row>
-    <row r="42" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:5">
       <c r="A42" s="1" t="s">
         <v>853</v>
       </c>
@@ -39017,7 +39021,7 @@
         <v>142</v>
       </c>
     </row>
-    <row r="43" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:5">
       <c r="A43" s="1" t="s">
         <v>869</v>
       </c>
@@ -39034,7 +39038,7 @@
         <v>477</v>
       </c>
     </row>
-    <row r="44" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:5">
       <c r="A44" s="1" t="s">
         <v>887</v>
       </c>
@@ -39051,7 +39055,7 @@
         <v>762</v>
       </c>
     </row>
-    <row r="45" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:5">
       <c r="A45" s="1" t="s">
         <v>904</v>
       </c>
@@ -39068,7 +39072,7 @@
         <v>915</v>
       </c>
     </row>
-    <row r="46" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:5">
       <c r="A46" s="1" t="s">
         <v>921</v>
       </c>
@@ -39085,7 +39089,7 @@
         <v>232</v>
       </c>
     </row>
-    <row r="47" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:5">
       <c r="A47" s="1" t="s">
         <v>938</v>
       </c>
@@ -39102,7 +39106,7 @@
         <v>433</v>
       </c>
     </row>
-    <row r="48" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:5">
       <c r="A48" s="1" t="s">
         <v>954</v>
       </c>
@@ -39119,7 +39123,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="49" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:5">
       <c r="A49" s="1" t="s">
         <v>971</v>
       </c>
@@ -39136,7 +39140,7 @@
         <v>984</v>
       </c>
     </row>
-    <row r="50" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:5">
       <c r="A50" s="1" t="s">
         <v>991</v>
       </c>
@@ -39153,7 +39157,7 @@
         <v>297</v>
       </c>
     </row>
-    <row r="51" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:5">
       <c r="A51" s="1" t="s">
         <v>1008</v>
       </c>
@@ -39170,7 +39174,7 @@
         <v>341</v>
       </c>
     </row>
-    <row r="52" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:5">
       <c r="A52" s="1" t="s">
         <v>1025</v>
       </c>
@@ -39187,7 +39191,7 @@
         <v>363</v>
       </c>
     </row>
-    <row r="53" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:5">
       <c r="A53" s="1" t="s">
         <v>1042</v>
       </c>
@@ -39204,7 +39208,7 @@
         <v>211</v>
       </c>
     </row>
-    <row r="54" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:5">
       <c r="A54" s="1" t="s">
         <v>1062</v>
       </c>
@@ -39221,7 +39225,7 @@
         <v>119</v>
       </c>
     </row>
-    <row r="55" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:5">
       <c r="A55" s="1" t="s">
         <v>1080</v>
       </c>
@@ -39238,7 +39242,7 @@
         <v>189</v>
       </c>
     </row>
-    <row r="56" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:5">
       <c r="A56" s="1" t="s">
         <v>1099</v>
       </c>
@@ -39255,7 +39259,7 @@
         <v>254</v>
       </c>
     </row>
-    <row r="57" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:5">
       <c r="A57" s="1" t="s">
         <v>1116</v>
       </c>
@@ -39272,7 +39276,7 @@
         <v>1128</v>
       </c>
     </row>
-    <row r="58" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:5">
       <c r="A58" s="1" t="s">
         <v>1135</v>
       </c>
@@ -39289,7 +39293,7 @@
         <v>386</v>
       </c>
     </row>
-    <row r="59" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:5">
       <c r="A59" s="1" t="s">
         <v>1155</v>
       </c>
@@ -39306,7 +39310,7 @@
         <v>1167</v>
       </c>
     </row>
-    <row r="60" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="60" spans="1:5">
       <c r="A60" s="1" t="s">
         <v>1174</v>
       </c>
@@ -39323,7 +39327,7 @@
         <v>539</v>
       </c>
     </row>
-    <row r="61" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="61" spans="1:5">
       <c r="A61" s="1" t="s">
         <v>1193</v>
       </c>
@@ -39340,7 +39344,7 @@
         <v>410</v>
       </c>
     </row>
-    <row r="62" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="62" spans="1:5">
       <c r="A62" s="1" t="s">
         <v>1212</v>
       </c>
@@ -39357,7 +39361,7 @@
         <v>232</v>
       </c>
     </row>
-    <row r="63" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="63" spans="1:5">
       <c r="A63" s="1" t="s">
         <v>1228</v>
       </c>
@@ -39374,7 +39378,7 @@
         <v>762</v>
       </c>
     </row>
-    <row r="64" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="64" spans="1:5">
       <c r="A64" s="1" t="s">
         <v>1247</v>
       </c>
@@ -39391,7 +39395,7 @@
         <v>1260</v>
       </c>
     </row>
-    <row r="65" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="65" spans="1:5">
       <c r="A65" s="1" t="s">
         <v>1267</v>
       </c>
@@ -39408,7 +39412,7 @@
         <v>189</v>
       </c>
     </row>
-    <row r="66" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="66" spans="1:5">
       <c r="A66" s="1" t="s">
         <v>1284</v>
       </c>
@@ -39425,7 +39429,7 @@
         <v>433</v>
       </c>
     </row>
-    <row r="67" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="67" spans="1:5">
       <c r="A67" s="1" t="s">
         <v>1302</v>
       </c>
@@ -39442,7 +39446,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="68" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="68" spans="1:5">
       <c r="A68" s="1" t="s">
         <v>1319</v>
       </c>
@@ -39459,7 +39463,7 @@
         <v>539</v>
       </c>
     </row>
-    <row r="69" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="69" spans="1:5">
       <c r="A69" s="1" t="s">
         <v>1338</v>
       </c>
@@ -39476,7 +39480,7 @@
         <v>984</v>
       </c>
     </row>
-    <row r="70" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="70" spans="1:5">
       <c r="A70" s="1" t="s">
         <v>1358</v>
       </c>
@@ -39493,7 +39497,7 @@
         <v>386</v>
       </c>
     </row>
-    <row r="71" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="71" spans="1:5">
       <c r="A71" s="1" t="s">
         <v>1375</v>
       </c>
@@ -39510,7 +39514,7 @@
         <v>1128</v>
       </c>
     </row>
-    <row r="72" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="72" spans="1:5">
       <c r="A72" s="1" t="s">
         <v>1392</v>
       </c>
@@ -39527,7 +39531,7 @@
         <v>915</v>
       </c>
     </row>
-    <row r="73" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="73" spans="1:5">
       <c r="A73" s="1" t="s">
         <v>1409</v>
       </c>
@@ -39544,7 +39548,7 @@
         <v>341</v>
       </c>
     </row>
-    <row r="74" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="74" spans="1:5">
       <c r="A74" s="1" t="s">
         <v>1427</v>
       </c>
@@ -39561,7 +39565,7 @@
         <v>297</v>
       </c>
     </row>
-    <row r="75" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="75" spans="1:5">
       <c r="A75" s="1" t="s">
         <v>1442</v>
       </c>
@@ -39578,7 +39582,7 @@
         <v>410</v>
       </c>
     </row>
-    <row r="76" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="76" spans="1:5">
       <c r="A76" s="1" t="s">
         <v>1457</v>
       </c>
@@ -39595,7 +39599,7 @@
         <v>254</v>
       </c>
     </row>
-    <row r="77" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="77" spans="1:5">
       <c r="A77" s="1" t="s">
         <v>1474</v>
       </c>
@@ -39612,7 +39616,7 @@
         <v>539</v>
       </c>
     </row>
-    <row r="78" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="78" spans="1:5">
       <c r="A78" s="1" t="s">
         <v>1492</v>
       </c>
@@ -39629,7 +39633,7 @@
         <v>477</v>
       </c>
     </row>
-    <row r="79" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="79" spans="1:5">
       <c r="A79" s="1" t="s">
         <v>1508</v>
       </c>
@@ -39646,7 +39650,7 @@
         <v>1167</v>
       </c>
     </row>
-    <row r="80" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="80" spans="1:5">
       <c r="A80" s="1" t="s">
         <v>1523</v>
       </c>
@@ -39663,7 +39667,7 @@
         <v>1128</v>
       </c>
     </row>
-    <row r="81" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="81" spans="1:5">
       <c r="A81" s="1" t="s">
         <v>1538</v>
       </c>
@@ -39680,7 +39684,7 @@
         <v>119</v>
       </c>
     </row>
-    <row r="82" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="82" spans="1:5">
       <c r="A82" s="1" t="s">
         <v>1557</v>
       </c>
@@ -39697,7 +39701,7 @@
         <v>142</v>
       </c>
     </row>
-    <row r="83" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="83" spans="1:5">
       <c r="A83" s="1" t="s">
         <v>1574</v>
       </c>
@@ -39716,6 +39720,6 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295"/>
 </worksheet>
 </file>
</xml_diff>